<commit_message>
Update Stock Analysis Data file: modify content for improved financial analysis
</commit_message>
<xml_diff>
--- a/stock_information_data/Stock_Analysis_Data.xlsx
+++ b/stock_information_data/Stock_Analysis_Data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aspire5 15 i7 4G2050\marketflow\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aspire5 15 i7 4G2050\marketflow\stock_information_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3AF53A33-4F74-42AF-924E-E4888657B021}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36CD4C20-A331-422A-9C69-13AE4C95F880}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="226" firstSheet="1" activeTab="1" xr2:uid="{25A1E8A8-8B79-4D62-AF4C-E3957BC49F2B}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="226" xr2:uid="{25A1E8A8-8B79-4D62-AF4C-E3957BC49F2B}"/>
   </bookViews>
   <sheets>
     <sheet name="Defense" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
       </extLst>
     </bk>
   </futureMetadata>
-  <futureMetadata name="XLRICHVALUE" count="144">
+  <futureMetadata name="XLRICHVALUE" count="145">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -328,745 +328,752 @@
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="118"/>
+          <xlrd:rvb i="116"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="121"/>
+          <xlrd:rvb i="119"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="124"/>
+          <xlrd:rvb i="122"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="127"/>
+          <xlrd:rvb i="125"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="130"/>
+          <xlrd:rvb i="128"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="133"/>
+          <xlrd:rvb i="131"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="136"/>
+          <xlrd:rvb i="134"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="139"/>
+          <xlrd:rvb i="137"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="142"/>
+          <xlrd:rvb i="140"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="144"/>
+          <xlrd:rvb i="143"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="147"/>
+          <xlrd:rvb i="145"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="150"/>
+          <xlrd:rvb i="148"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="153"/>
+          <xlrd:rvb i="151"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="156"/>
+          <xlrd:rvb i="154"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="159"/>
+          <xlrd:rvb i="157"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="162"/>
+          <xlrd:rvb i="160"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="165"/>
+          <xlrd:rvb i="163"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="168"/>
+          <xlrd:rvb i="166"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="171"/>
+          <xlrd:rvb i="169"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="174"/>
+          <xlrd:rvb i="172"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="176"/>
+          <xlrd:rvb i="175"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="179"/>
+          <xlrd:rvb i="177"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="182"/>
+          <xlrd:rvb i="180"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="185"/>
+          <xlrd:rvb i="183"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="187"/>
+          <xlrd:rvb i="186"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="190"/>
+          <xlrd:rvb i="188"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="192"/>
+          <xlrd:rvb i="191"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="195"/>
+          <xlrd:rvb i="193"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="198"/>
+          <xlrd:rvb i="196"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="201"/>
+          <xlrd:rvb i="199"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="204"/>
+          <xlrd:rvb i="202"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="207"/>
+          <xlrd:rvb i="205"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="210"/>
+          <xlrd:rvb i="208"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="213"/>
+          <xlrd:rvb i="211"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="216"/>
+          <xlrd:rvb i="214"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="222"/>
+          <xlrd:rvb i="217"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="225"/>
+          <xlrd:rvb i="223"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="228"/>
+          <xlrd:rvb i="226"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="231"/>
+          <xlrd:rvb i="229"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="234"/>
+          <xlrd:rvb i="232"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="237"/>
+          <xlrd:rvb i="235"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="240"/>
+          <xlrd:rvb i="238"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="243"/>
+          <xlrd:rvb i="241"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="246"/>
+          <xlrd:rvb i="244"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="249"/>
+          <xlrd:rvb i="247"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="252"/>
+          <xlrd:rvb i="250"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="255"/>
+          <xlrd:rvb i="253"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="258"/>
+          <xlrd:rvb i="256"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="261"/>
+          <xlrd:rvb i="259"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="264"/>
+          <xlrd:rvb i="262"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="267"/>
+          <xlrd:rvb i="265"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="270"/>
+          <xlrd:rvb i="268"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="273"/>
+          <xlrd:rvb i="271"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="276"/>
+          <xlrd:rvb i="274"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="279"/>
+          <xlrd:rvb i="277"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="282"/>
+          <xlrd:rvb i="280"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="285"/>
+          <xlrd:rvb i="283"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="287"/>
+          <xlrd:rvb i="286"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="289"/>
+          <xlrd:rvb i="288"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="292"/>
+          <xlrd:rvb i="290"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="295"/>
+          <xlrd:rvb i="293"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="298"/>
+          <xlrd:rvb i="296"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="301"/>
+          <xlrd:rvb i="299"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="304"/>
+          <xlrd:rvb i="302"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="307"/>
+          <xlrd:rvb i="305"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="310"/>
+          <xlrd:rvb i="308"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="313"/>
+          <xlrd:rvb i="311"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="316"/>
+          <xlrd:rvb i="314"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="319"/>
+          <xlrd:rvb i="317"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="322"/>
+          <xlrd:rvb i="320"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="325"/>
+          <xlrd:rvb i="323"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="328"/>
+          <xlrd:rvb i="326"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="331"/>
+          <xlrd:rvb i="329"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="334"/>
+          <xlrd:rvb i="332"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="337"/>
+          <xlrd:rvb i="335"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="340"/>
+          <xlrd:rvb i="338"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="343"/>
+          <xlrd:rvb i="341"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="346"/>
+          <xlrd:rvb i="344"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="348"/>
+          <xlrd:rvb i="347"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="351"/>
+          <xlrd:rvb i="349"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="353"/>
+          <xlrd:rvb i="352"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="356"/>
+          <xlrd:rvb i="354"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="359"/>
+          <xlrd:rvb i="357"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="362"/>
+          <xlrd:rvb i="360"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="365"/>
+          <xlrd:rvb i="363"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="368"/>
+          <xlrd:rvb i="366"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="371"/>
+          <xlrd:rvb i="369"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="374"/>
+          <xlrd:rvb i="372"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="377"/>
+          <xlrd:rvb i="375"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="380"/>
+          <xlrd:rvb i="378"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="383"/>
+          <xlrd:rvb i="381"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="385"/>
+          <xlrd:rvb i="384"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="387"/>
+          <xlrd:rvb i="386"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="390"/>
+          <xlrd:rvb i="388"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="393"/>
+          <xlrd:rvb i="391"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="396"/>
+          <xlrd:rvb i="394"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="399"/>
+          <xlrd:rvb i="397"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="402"/>
+          <xlrd:rvb i="400"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="405"/>
+          <xlrd:rvb i="403"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="408"/>
+          <xlrd:rvb i="406"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="410"/>
+          <xlrd:rvb i="409"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="413"/>
+          <xlrd:rvb i="411"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="415"/>
+          <xlrd:rvb i="414"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="417"/>
+          <xlrd:rvb i="416"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="420"/>
+          <xlrd:rvb i="418"/>
         </ext>
       </extLst>
     </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="421"/>
+        </ext>
+      </extLst>
+    </bk>
   </futureMetadata>
   <cellMetadata count="1">
     <bk>
       <rc t="1" v="0"/>
     </bk>
   </cellMetadata>
-  <valueMetadata count="144">
+  <valueMetadata count="145">
     <bk>
       <rc t="2" v="0"/>
     </bk>
@@ -1498,13 +1505,16 @@
     </bk>
     <bk>
       <rc t="2" v="143"/>
+    </bk>
+    <bk>
+      <rc t="2" v="144"/>
     </bk>
   </valueMetadata>
 </metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="308">
   <si>
     <t>General Electric Company</t>
   </si>
@@ -2425,6 +2435,9 @@
   </si>
   <si>
     <t>Shares Outstanding</t>
+  </si>
+  <si>
+    <t>Stock Symbol</t>
   </si>
 </sst>
 </file>
@@ -2568,7 +2581,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2623,7 +2636,7 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2638,8 +2651,8 @@
     <xf numFmtId="3" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2661,6 +2674,9 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="10" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2791,7 +2807,7 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="421">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="422">
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1tr1h&amp;q=XNYS%3aGE&amp;form=skydnc</v>
     <v>Learn more on Bing</v>
@@ -3101,7 +3117,7 @@
     <v>NORTHROP GRUMMAN CORPORATION</v>
     <v>NORTHROP GRUMMAN CORPORATION</v>
     <v>599.79</v>
-    <v>23.3643</v>
+    <v>23.552399999999999</v>
     <v>597.21</v>
     <v>592.44000000000005</v>
     <v>592.46</v>
@@ -4122,9 +4138,9 @@
     <v>17.34</v>
     <v>1.4850000000000001</v>
     <v>0.5</v>
-    <v>-6.4480000000000006E-3</v>
+    <v>0</v>
     <v>1.8600999999999999E-2</v>
-    <v>-0.17649999999999999</v>
+    <v>0</v>
     <v>USD</v>
     <v>CAE Inc. is a technology company. It operates in two segments: Civil Aviation and Defense and Security. The Civil Aviation training segment provides comprehensive training solutions for flight, cabin, maintenance and ground personnel in commercial, business and helicopter aviation, a complete range of flight simulation training devices, ab initio pilot training and crew sourcing services, as well as aircraft flight operations solutions. It manages approximately 324 full-flight simulators. Its training systems includes CAE Real-time Insights and Standardized Evaluations (CAE Rise), which improves training through the integration of untapped flight and simulator data-driven insights into training. The Defense and Security segment provides platform-independent training and simulation solutions, preparing global defense and security forces for the mission ahead. In addition to solutions delivered to customer sites, it provides comprehensive training at its CAE global training centers.</v>
     <v>13000</v>
@@ -4142,10 +4158,10 @@
     <v>CAE Inc.</v>
     <v>CAE Inc.</v>
     <v>27.05</v>
-    <v>29.264600000000002</v>
+    <v>28.729600000000001</v>
     <v>26.88</v>
     <v>27.38</v>
-    <v>27.203499999999998</v>
+    <v>27.38</v>
     <v>320726200</v>
     <v>CAE</v>
     <v>CAE Inc. (XNYS:CAE)</v>
@@ -4844,6 +4860,11 @@
     <v>Shares outstanding</v>
     <v>0</v>
   </rv>
+  <rv s="10">
+    <v>12</v>
+    <v>Ticker symbol</v>
+    <v>0</v>
+  </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=c432pr&amp;q=XNAS%3aIPAX&amp;form=skydnc</v>
     <v>Learn more on Bing</v>
@@ -4878,7 +4899,7 @@
     <v>Aerospace &amp; Defense</v>
     <v>Stock</v>
     <v>45891.99947790469</v>
-    <v>116</v>
+    <v>117</v>
     <v>8.52</v>
     <v>1602214000</v>
     <v>INTUITIVE MACHINES, INC.</v>
@@ -4896,7 +4917,7 @@
     <v>2023</v>
   </rv>
   <rv s="2">
-    <v>117</v>
+    <v>118</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=bxcpvh&amp;q=XNYS%3aEVEX&amp;form=skydnc</v>
@@ -4932,7 +4953,7 @@
     <v>Aerospace &amp; Defense</v>
     <v>Stock</v>
     <v>45891.991145057815</v>
-    <v>119</v>
+    <v>120</v>
     <v>3.86</v>
     <v>1391596882</v>
     <v>Eve Holding, Inc.</v>
@@ -4949,7 +4970,7 @@
     <v>2020</v>
   </rv>
   <rv s="2">
-    <v>120</v>
+    <v>121</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1qthw&amp;q=XNYS%3aDCO&amp;form=skydnc</v>
@@ -4985,7 +5006,7 @@
     <v>Aerospace &amp; Defense</v>
     <v>Stock</v>
     <v>45891.958333367969</v>
-    <v>122</v>
+    <v>123</v>
     <v>89.9</v>
     <v>1385520021</v>
     <v>DUCOMMUN INCORPORATED</v>
@@ -5003,7 +5024,7 @@
     <v>1970</v>
   </rv>
   <rv s="2">
-    <v>123</v>
+    <v>124</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=bt7jw7&amp;q=XNAS%3aEH&amp;form=skydnc</v>
@@ -5039,7 +5060,7 @@
     <v>Aerospace &amp; Defense</v>
     <v>Stock</v>
     <v>45891.999759964841</v>
-    <v>125</v>
+    <v>126</v>
     <v>18.035</v>
     <v>1332439758</v>
     <v>EHang Holdings Limited</v>
@@ -5057,7 +5078,7 @@
     <v>2014</v>
   </rv>
   <rv s="2">
-    <v>126</v>
+    <v>127</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=bxe2w7&amp;q=XNYS%3aRDW&amp;form=skydnc</v>
@@ -5093,7 +5114,7 @@
     <v>Aerospace &amp; Defense</v>
     <v>Stock</v>
     <v>45891.99905558984</v>
-    <v>128</v>
+    <v>129</v>
     <v>8.61</v>
     <v>1310764000</v>
     <v>REDWIRE CORPORATION</v>
@@ -5110,7 +5131,7 @@
     <v>2021</v>
   </rv>
   <rv s="2">
-    <v>129</v>
+    <v>130</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1nx1h&amp;q=XNAS%3aATRO&amp;form=skydnc</v>
@@ -5146,7 +5167,7 @@
     <v>Aerospace &amp; Defense</v>
     <v>Stock</v>
     <v>45891.974236376562</v>
-    <v>131</v>
+    <v>132</v>
     <v>35.61</v>
     <v>1269420000</v>
     <v>ASTRONICS CORPORATION</v>
@@ -5164,7 +5185,7 @@
     <v>1968</v>
   </rv>
   <rv s="2">
-    <v>132</v>
+    <v>133</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=c3yrjc&amp;q=XNYS%3aCDRE&amp;form=skydnc</v>
@@ -5200,7 +5221,7 @@
     <v>Aerospace &amp; Defense</v>
     <v>Stock</v>
     <v>45891.958333356248</v>
-    <v>134</v>
+    <v>135</v>
     <v>29.87</v>
     <v>1263019000</v>
     <v>CADRE HOLDINGS, INC.</v>
@@ -5218,7 +5239,7 @@
     <v>2012</v>
   </rv>
   <rv s="2">
-    <v>135</v>
+    <v>136</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a2y55r&amp;q=XNAS%3aRCAT&amp;form=skydnc</v>
@@ -5254,7 +5275,7 @@
     <v>Aerospace &amp; Defense</v>
     <v>Stock</v>
     <v>45891.999939872658</v>
-    <v>137</v>
+    <v>138</v>
     <v>9.51</v>
     <v>979685033</v>
     <v>RED CAT HOLDINGS, INC.</v>
@@ -5272,7 +5293,7 @@
     <v>2001</v>
   </rv>
   <rv s="2">
-    <v>138</v>
+    <v>139</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1yofr&amp;q=XNYS%3aNPK&amp;form=skydnc</v>
@@ -5308,7 +5329,7 @@
     <v>Aerospace &amp; Defense</v>
     <v>Stock</v>
     <v>45891.958333344533</v>
-    <v>140</v>
+    <v>141</v>
     <v>103.66</v>
     <v>785661851</v>
     <v>NATIONAL PRESTO INDUSTRIES, INC.</v>
@@ -5326,7 +5347,7 @@
     <v>1905</v>
   </rv>
   <rv s="2">
-    <v>141</v>
+    <v>142</v>
   </rv>
   <rv s="7">
     <v>en-AE</v>
@@ -5375,7 +5396,7 @@
     <v>2021</v>
   </rv>
   <rv s="2">
-    <v>143</v>
+    <v>144</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a21yu2&amp;q=XNYS%3aRGR&amp;form=skydnc</v>
@@ -5411,7 +5432,7 @@
     <v>Leisure Products</v>
     <v>Stock</v>
     <v>45891.959160786719</v>
-    <v>145</v>
+    <v>146</v>
     <v>34.020000000000003</v>
     <v>564216500</v>
     <v>STURM, RUGER &amp; COMPANY, INC.</v>
@@ -5429,7 +5450,7 @@
     <v>1969</v>
   </rv>
   <rv s="2">
-    <v>146</v>
+    <v>147</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=bwo5nm&amp;q=XNYS%3aEVTL&amp;form=skydnc</v>
@@ -5465,7 +5486,7 @@
     <v>Aerospace &amp; Defense</v>
     <v>Stock</v>
     <v>45891.999646816403</v>
-    <v>148</v>
+    <v>149</v>
     <v>4.7149999999999999</v>
     <v>511099366</v>
     <v>VERTICAL AEROSPACE LTD.</v>
@@ -5482,7 +5503,7 @@
     <v>2021</v>
   </rv>
   <rv s="2">
-    <v>149</v>
+    <v>150</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a23yh7&amp;q=XNAS%3aTATT&amp;form=skydnc</v>
@@ -5518,7 +5539,7 @@
     <v>Machinery, Equipment &amp; Components</v>
     <v>Stock</v>
     <v>45891.950210798437</v>
-    <v>151</v>
+    <v>152</v>
     <v>35.01</v>
     <v>476989600</v>
     <v>TAT TECHNOLOGIES LTD.</v>
@@ -5536,7 +5557,7 @@
     <v>1985</v>
   </rv>
   <rv s="2">
-    <v>152</v>
+    <v>153</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a2v5hw&amp;q=XNAS%3aBYRN&amp;form=skydnc</v>
@@ -5572,7 +5593,7 @@
     <v>Aerospace &amp; Defense</v>
     <v>Stock</v>
     <v>45891.988739490625</v>
-    <v>154</v>
+    <v>155</v>
     <v>19.133199999999999</v>
     <v>458616962</v>
     <v>BYRNA TECHNOLOGIES INC.</v>
@@ -5590,7 +5611,7 @@
     <v>2005</v>
   </rv>
   <rv s="2">
-    <v>155</v>
+    <v>156</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1zx77&amp;q=XNYS%3aPKE&amp;form=skydnc</v>
@@ -5626,7 +5647,7 @@
     <v>Aerospace &amp; Defense</v>
     <v>Stock</v>
     <v>45891.989026075782</v>
-    <v>157</v>
+    <v>158</v>
     <v>18.100000000000001</v>
     <v>378253752</v>
     <v>PARK AEROSPACE CORP.</v>
@@ -5644,7 +5665,7 @@
     <v>1954</v>
   </rv>
   <rv s="2">
-    <v>158</v>
+    <v>159</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=c1b4z2&amp;q=XNAS%3aSATL&amp;form=skydnc</v>
@@ -5680,7 +5701,7 @@
     <v>Metals &amp; Mining</v>
     <v>Stock</v>
     <v>45891.999934039064</v>
-    <v>160</v>
+    <v>161</v>
     <v>3.4350000000000001</v>
     <v>370544733</v>
     <v>Satellogic Inc.</v>
@@ -5698,7 +5719,7 @@
     <v>2021</v>
   </rv>
   <rv s="2">
-    <v>161</v>
+    <v>162</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1nk27&amp;q=XNAS%3aSWBI&amp;form=skydnc</v>
@@ -5734,7 +5755,7 @@
     <v>Aerospace &amp; Defense</v>
     <v>Stock</v>
     <v>45891.991994478907</v>
-    <v>163</v>
+    <v>164</v>
     <v>7.9850000000000003</v>
     <v>364674400</v>
     <v>SMITH &amp; WESSON BRANDS, INC.</v>
@@ -5752,7 +5773,7 @@
     <v>1991</v>
   </rv>
   <rv s="2">
-    <v>164</v>
+    <v>165</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1vtcw&amp;q=XNAS%3aISSC&amp;form=skydnc</v>
@@ -5788,7 +5809,7 @@
     <v>Aerospace &amp; Defense</v>
     <v>Stock</v>
     <v>45891.994240022657</v>
-    <v>166</v>
+    <v>167</v>
     <v>13.477600000000001</v>
     <v>250848716</v>
     <v>INNOVATIVE SOLUTIONS AND SUPPORT, INC.</v>
@@ -5806,7 +5827,7 @@
     <v>1988</v>
   </rv>
   <rv s="2">
-    <v>167</v>
+    <v>168</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1vpr7&amp;q=XNYS%3aSPCE&amp;form=skydnc</v>
@@ -5828,9 +5849,9 @@
     <v>2.1800000000000002</v>
     <v>2.1286999999999998</v>
     <v>0.16</v>
-    <v>-3.2060000000000001E-3</v>
+    <v>-6.3490000000000005E-3</v>
     <v>5.3512000000000004E-2</v>
-    <v>-1.01E-2</v>
+    <v>-0.02</v>
     <v>USD</v>
     <v>Virgin Galactic Holdings, Inc. is an aerospace and space travel company, which offers access to space for private individuals, researchers, and government agencies. The Company’s operations include design and development, manufacturing, ground and flight testing, and post-flight maintenance of its spaceflight system vehicles. The Company has developed a portfolio of proprietary technologies that are embodied in the specialized vehicles that it has created to enable commercial spaceflight. These technologies underpin its carrier aircraft, the mothership; its spaceships; its hybrid rocket motor; and its safety systems. Its Carrier Aircraft-The mothership is a twin-fuselage, custom-built aircraft designed to carry spaceships up to an altitude of approximately 45,000 feet, where the spaceship is released for its flight into space. Its Virgin Galactic spaceships are reusable with the capacity to carry pilots and private astronauts, research experiments and researchers.</v>
     <v>744</v>
@@ -5842,7 +5863,7 @@
     <v>Aerospace &amp; Defense</v>
     <v>Stock</v>
     <v>45891.998493125</v>
-    <v>169</v>
+    <v>170</v>
     <v>2.99</v>
     <v>181411500</v>
     <v>VIRGIN GALACTIC HOLDINGS, INC.</v>
@@ -5850,7 +5871,7 @@
     <v>3.05</v>
     <v>2.99</v>
     <v>3.15</v>
-    <v>3.1398999999999999</v>
+    <v>3.13</v>
     <v>57590960</v>
     <v>SPCE</v>
     <v>VIRGIN GALACTIC HOLDINGS, INC. (XNYS:SPCE)</v>
@@ -5859,7 +5880,7 @@
     <v>2019</v>
   </rv>
   <rv s="2">
-    <v>170</v>
+    <v>171</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a2skar&amp;q=XNAS%3aPOWW&amp;form=skydnc</v>
@@ -5895,7 +5916,7 @@
     <v>Leisure Products</v>
     <v>Stock</v>
     <v>45891.952196851562</v>
-    <v>172</v>
+    <v>173</v>
     <v>1.3935</v>
     <v>173324000</v>
     <v>OUTDOOR HOLDING COMPANY</v>
@@ -5913,7 +5934,7 @@
     <v>2016</v>
   </rv>
   <rv s="2">
-    <v>173</v>
+    <v>174</v>
   </rv>
   <rv s="11">
     <v>en-AE</v>
@@ -5961,7 +5982,7 @@
     <v>2021</v>
   </rv>
   <rv s="2">
-    <v>175</v>
+    <v>176</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=bstrec&amp;q=XNAS%3aDPRO&amp;form=skydnc</v>
@@ -5997,7 +6018,7 @@
     <v>Aerospace &amp; Defense</v>
     <v>Stock</v>
     <v>45891.999758553124</v>
-    <v>177</v>
+    <v>178</v>
     <v>4.0250000000000004</v>
     <v>101537400</v>
     <v>DRAGANFLY INC</v>
@@ -6015,7 +6036,7 @@
     <v>2018</v>
   </rv>
   <rv s="2">
-    <v>178</v>
+    <v>179</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1q352&amp;q=XNAS%3aCODA&amp;form=skydnc</v>
@@ -6051,7 +6072,7 @@
     <v>Electronic Equipment &amp; Parts</v>
     <v>Stock</v>
     <v>45891.840328263279</v>
-    <v>180</v>
+    <v>181</v>
     <v>7.26</v>
     <v>85266410</v>
     <v>CODA OCTOPUS GROUP, INC.</v>
@@ -6069,7 +6090,7 @@
     <v>2004</v>
   </rv>
   <rv s="2">
-    <v>181</v>
+    <v>182</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a2r8fr&amp;q=OTCM%3aOPXS&amp;form=skydnc</v>
@@ -6105,7 +6126,7 @@
     <v>Aerospace &amp; Defense</v>
     <v>Stock</v>
     <v>45891.867851099218</v>
-    <v>183</v>
+    <v>184</v>
     <v>10.1</v>
     <v>71901680</v>
     <v>OPTEX SYSTEMS HOLDINGS, INC.</v>
@@ -6123,7 +6144,7 @@
     <v>2006</v>
   </rv>
   <rv s="2">
-    <v>184</v>
+    <v>185</v>
   </rv>
   <rv s="7">
     <v>en-AE</v>
@@ -6172,7 +6193,7 @@
     <v>2024</v>
   </rv>
   <rv s="2">
-    <v>186</v>
+    <v>187</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a22y52&amp;q=XNYS%3aSIF&amp;form=skydnc</v>
@@ -6208,7 +6229,7 @@
     <v>Metals &amp; Mining</v>
     <v>Stock</v>
     <v>45892.000000034372</v>
-    <v>188</v>
+    <v>189</v>
     <v>6.6101000000000001</v>
     <v>43880769</v>
     <v>SIFCO INDUSTRIES, INC</v>
@@ -6225,7 +6246,7 @@
     <v>1916</v>
   </rv>
   <rv s="2">
-    <v>189</v>
+    <v>190</v>
   </rv>
   <rv s="12">
     <v>en-AE</v>
@@ -6272,7 +6293,7 @@
     <v>2017</v>
   </rv>
   <rv s="2">
-    <v>191</v>
+    <v>192</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1vlim&amp;q=XNAS%3aINPX&amp;form=skydnc</v>
@@ -6308,7 +6329,7 @@
     <v>Aerospace &amp; Defense</v>
     <v>Stock</v>
     <v>45891.998462892967</v>
-    <v>193</v>
+    <v>194</v>
     <v>1.71</v>
     <v>34835700</v>
     <v>XTI AEROSPACE, INC.</v>
@@ -6326,7 +6347,7 @@
     <v>1999</v>
   </rv>
   <rv s="2">
-    <v>194</v>
+    <v>195</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=c2ytlh&amp;q=XNAS%3aCLAQ&amp;form=skydnc</v>
@@ -6362,7 +6383,7 @@
     <v>Machinery, Equipment &amp; Components</v>
     <v>Stock</v>
     <v>45891.99685263828</v>
-    <v>196</v>
+    <v>197</v>
     <v>0.79</v>
     <v>34519980</v>
     <v>Nauticus Robotics, Inc.</v>
@@ -6380,7 +6401,7 @@
     <v>2020</v>
   </rv>
   <rv s="2">
-    <v>197</v>
+    <v>198</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1qltc&amp;q=OTCM%3aCVUA&amp;form=skydnc</v>
@@ -6416,7 +6437,7 @@
     <v>Aerospace &amp; Defense</v>
     <v>Stock</v>
     <v>45891.976637407031</v>
-    <v>199</v>
+    <v>200</v>
     <v>2.5720000000000001</v>
     <v>33515070</v>
     <v>CPI AEROSTRUCTURES, INC.</v>
@@ -6433,7 +6454,7 @@
     <v>1980</v>
   </rv>
   <rv s="2">
-    <v>200</v>
+    <v>201</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=c4ipvh&amp;q=XNAS%3aSIDU&amp;form=skydnc</v>
@@ -6469,7 +6490,7 @@
     <v>Aerospace &amp; Defense</v>
     <v>Stock</v>
     <v>45891.994755416403</v>
-    <v>202</v>
+    <v>203</v>
     <v>1.1499999999999999</v>
     <v>30028030</v>
     <v>SIDUS SPACE, INC.</v>
@@ -6487,7 +6508,7 @@
     <v>2021</v>
   </rv>
   <rv s="2">
-    <v>203</v>
+    <v>204</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=c6q7vh&amp;q=XNAS%3aPRZO&amp;form=skydnc</v>
@@ -6522,7 +6543,7 @@
     <v>Aerospace &amp; Defense</v>
     <v>Stock</v>
     <v>45891.99636075156</v>
-    <v>205</v>
+    <v>206</v>
     <v>1.38</v>
     <v>26831990</v>
     <v>PARAZERO TECHNOLOGIES LTD</v>
@@ -6540,7 +6561,7 @@
     <v>2013</v>
   </rv>
   <rv s="2">
-    <v>206</v>
+    <v>207</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1r9im&amp;q=XNYS%3aNILE&amp;form=skydnc</v>
@@ -6576,7 +6597,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.997866735939</v>
-    <v>208</v>
+    <v>209</v>
     <v>0.56320000000000003</v>
     <v>18933080</v>
     <v>HYPERSCALE DATA, INC.</v>
@@ -6593,7 +6614,7 @@
     <v>2017</v>
   </rv>
   <rv s="2">
-    <v>209</v>
+    <v>210</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=btdivh&amp;q=XNAS%3aMNTS&amp;form=skydnc</v>
@@ -6615,9 +6636,9 @@
     <v>1.03</v>
     <v>1.1438999999999999</v>
     <v>0.17</v>
-    <v>-1.3172E-2</v>
+    <v>6.7589999999999994E-3</v>
     <v>0.13281299999999999</v>
-    <v>-1.9099999999999999E-2</v>
+    <v>9.7999999999999997E-3</v>
     <v>USD</v>
     <v>Momentus Inc. is a commercial space company. The Company offers satellites, satellite buses, and other satellite components, transportation and infrastructure services, including hosted payloads and other in-orbit services to help enable the commercialization of space. The Company offers satellites and satellite buses, and technology designed to meet the specific needs of government and commercial customers. It is focused on providing services including last-mile satellite transportation, payload-hosting, on-orbit satellite refueling, on-orbit inspection, on-orbit satellite maintenance, de-orbiting, debris removal, and other satellite-to-satellite service offerings. Its transportation service offering focuses on delivering its customers’ satellites to precision orbits. Its orbital service vehicles (OSVs) provide in-space services to its customers, including space transportation, payload hosting, and in-orbit servicing.</v>
     <v>24</v>
@@ -6629,7 +6650,7 @@
     <v>Aerospace &amp; Defense</v>
     <v>Stock</v>
     <v>45891.999949791403</v>
-    <v>211</v>
+    <v>212</v>
     <v>1.38</v>
     <v>16869830</v>
     <v>MOMENTUS INC.</v>
@@ -6638,7 +6659,7 @@
     <v>0</v>
     <v>1.28</v>
     <v>1.45</v>
-    <v>1.4309000000000001</v>
+    <v>1.4598</v>
     <v>11634370</v>
     <v>MNTS</v>
     <v>MOMENTUS INC. (XNAS:MNTS)</v>
@@ -6647,7 +6668,7 @@
     <v>2019</v>
   </rv>
   <rv s="2">
-    <v>212</v>
+    <v>213</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1n75r&amp;q=XNYS%3aAIRI&amp;form=skydnc</v>
@@ -6683,7 +6704,7 @@
     <v>Aerospace &amp; Defense</v>
     <v>Stock</v>
     <v>45891.91983267344</v>
-    <v>214</v>
+    <v>215</v>
     <v>3.01</v>
     <v>14840780</v>
     <v>AIR INDUSTRIES GROUP</v>
@@ -6700,7 +6721,7 @@
     <v>2013</v>
   </rv>
   <rv s="2">
-    <v>215</v>
+    <v>216</v>
   </rv>
   <rv s="0">
     <v>http://en.wikipedia.org/wiki/IBM</v>
@@ -6708,12 +6729,12 @@
   </rv>
   <rv s="4">
     <v>66</v>
-    <v>217</v>
+    <v>218</v>
   </rv>
   <rv s="5">
     <v>12</v>
     <v>https://www.bing.com/th?id=AMMS_41da901be1b295dc42c72dadb9c0f67d&amp;qlt=95</v>
-    <v>218</v>
+    <v>219</v>
     <v>0</v>
     <v>https://www.bing.com/images/search?form=xlimg&amp;q=ibm</v>
     <v>Image of INTERNATIONAL BUSINESS MACHINES CORPORATION</v>
@@ -6749,11 +6770,11 @@
     <v>XNYS</v>
     <v>One New Orchard Road, ARMONK, NY, 10504 US</v>
     <v>243.68</v>
-    <v>219</v>
+    <v>220</v>
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.999857858595</v>
-    <v>220</v>
+    <v>221</v>
     <v>240.22</v>
     <v>225511500000</v>
     <v>INTERNATIONAL BUSINESS MACHINES CORPORATION</v>
@@ -6771,7 +6792,7 @@
     <v>1911</v>
   </rv>
   <rv s="2">
-    <v>221</v>
+    <v>222</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1mthw&amp;q=XNYS%3aACN&amp;form=skydnc</v>
@@ -6807,7 +6828,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.995813900001</v>
-    <v>223</v>
+    <v>224</v>
     <v>254.4701</v>
     <v>161455876894</v>
     <v>ACCENTURE PUBLIC LIMITED COMPANY</v>
@@ -6825,7 +6846,7 @@
     <v>2009</v>
   </rv>
   <rv s="2">
-    <v>224</v>
+    <v>225</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1sx27&amp;q=XNAS%3aFISV&amp;form=skydnc</v>
@@ -6861,7 +6882,7 @@
     <v>Professional &amp; Commercial Services</v>
     <v>Stock</v>
     <v>45891.995430196097</v>
-    <v>226</v>
+    <v>227</v>
     <v>136.79</v>
     <v>75929098176</v>
     <v>FISERV, INC.</v>
@@ -6879,7 +6900,7 @@
     <v>1992</v>
   </rv>
   <rv s="2">
-    <v>227</v>
+    <v>228</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1vkgh&amp;q=XNYS%3aINFY&amp;form=skydnc</v>
@@ -6915,7 +6936,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.991217152347</v>
-    <v>229</v>
+    <v>230</v>
     <v>16.98</v>
     <v>70657770000</v>
     <v>INFOSYS LIMITED</v>
@@ -6933,7 +6954,7 @@
     <v>1981</v>
   </rv>
   <rv s="2">
-    <v>230</v>
+    <v>231</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1swsm&amp;q=XNYS%3aFIS&amp;form=skydnc</v>
@@ -6969,7 +6990,7 @@
     <v>Financial Technology (Fintech) &amp; Infrastructure</v>
     <v>Stock</v>
     <v>45891.991468228909</v>
-    <v>232</v>
+    <v>233</v>
     <v>69.924999999999997</v>
     <v>37485890000</v>
     <v>FIDELITY NATIONAL INFORMATION SERVICES, INC.</v>
@@ -6987,7 +7008,7 @@
     <v>2001</v>
   </rv>
   <rv s="2">
-    <v>233</v>
+    <v>234</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1qhz2&amp;q=XNAS%3aCTSH&amp;form=skydnc</v>
@@ -7023,13 +7044,13 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.966609212497</v>
-    <v>235</v>
+    <v>236</v>
     <v>71.38</v>
     <v>35345210000</v>
     <v>COGNIZANT TECHNOLOGY SOLUTIONS CORPORATION</v>
     <v>COGNIZANT TECHNOLOGY SOLUTIONS CORPORATION</v>
     <v>71.569999999999993</v>
-    <v>14.702199999999999</v>
+    <v>14.440300000000001</v>
     <v>71.08</v>
     <v>72.37</v>
     <v>72.989999999999995</v>
@@ -7041,7 +7062,7 @@
     <v>1988</v>
   </rv>
   <rv s="2">
-    <v>236</v>
+    <v>237</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1ossm&amp;q=XNYS%3aBR&amp;form=skydnc</v>
@@ -7077,7 +7098,7 @@
     <v>Professional &amp; Commercial Services</v>
     <v>Stock</v>
     <v>45891.974147117966</v>
-    <v>238</v>
+    <v>239</v>
     <v>260.80500000000001</v>
     <v>30708960000</v>
     <v>BROADRIDGE FINANCIAL SOLUTIONS, INC.</v>
@@ -7095,7 +7116,7 @@
     <v>2006</v>
   </rv>
   <rv s="2">
-    <v>239</v>
+    <v>240</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a25wh7&amp;q=XNYS%3aWIT&amp;form=skydnc</v>
@@ -7131,7 +7152,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.986764062502</v>
-    <v>241</v>
+    <v>242</v>
     <v>2.7650000000000001</v>
     <v>29835400000</v>
     <v>WIPRO LIMITED</v>
@@ -7149,7 +7170,7 @@
     <v>1945</v>
   </rv>
   <rv s="2">
-    <v>242</v>
+    <v>243</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1wt7w&amp;q=XNYS%3aLDOS&amp;form=skydnc</v>
@@ -7185,13 +7206,13 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.992521180466</v>
-    <v>244</v>
+    <v>245</v>
     <v>180.3</v>
     <v>23316760000</v>
     <v>LEIDOS HOLDINGS, INC.</v>
     <v>LEIDOS HOLDINGS, INC.</v>
     <v>180.5</v>
-    <v>17.237300000000001</v>
+    <v>17.114000000000001</v>
     <v>180.44</v>
     <v>181.74</v>
     <v>183.35</v>
@@ -7203,7 +7224,7 @@
     <v>2005</v>
   </rv>
   <rv s="2">
-    <v>245</v>
+    <v>246</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1pf4c&amp;q=XNAS%3aCDW&amp;form=skydnc</v>
@@ -7239,7 +7260,7 @@
     <v>Integrated Hardware &amp; Software</v>
     <v>Stock</v>
     <v>45891.989497048438</v>
-    <v>247</v>
+    <v>248</v>
     <v>164.27500000000001</v>
     <v>21887136900</v>
     <v>CDW CORPORATION</v>
@@ -7257,7 +7278,7 @@
     <v>2007</v>
   </rv>
   <rv s="2">
-    <v>248</v>
+    <v>249</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1tv4c&amp;q=XNYS%3aGIB&amp;form=skydnc</v>
@@ -7293,7 +7314,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.958333356248</v>
-    <v>250</v>
+    <v>251</v>
     <v>94.82</v>
     <v>29708370000</v>
     <v>CGI INC.</v>
@@ -7311,7 +7332,7 @@
     <v>1995</v>
   </rv>
   <rv s="2">
-    <v>251</v>
+    <v>252</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1vtoc&amp;q=XNYS%3aIT&amp;form=skydnc</v>
@@ -7347,7 +7368,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.987458414063</v>
-    <v>253</v>
+    <v>254</v>
     <v>245.04</v>
     <v>18926380000</v>
     <v>GARTNER, INC.</v>
@@ -7365,7 +7386,7 @@
     <v>1990</v>
   </rv>
   <rv s="2">
-    <v>254</v>
+    <v>255</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1w6zr&amp;q=XNAS%3aJKHY&amp;form=skydnc</v>
@@ -7401,7 +7422,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.872458853904</v>
-    <v>256</v>
+    <v>257</v>
     <v>163.72999999999999</v>
     <v>12055420000</v>
     <v>JACK HENRY &amp; ASSOCIATES, INC.</v>
@@ -7419,7 +7440,7 @@
     <v>1985</v>
   </rv>
   <rv s="2">
-    <v>257</v>
+    <v>258</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=c21yvh&amp;q=XNAS%3aAUR&amp;form=skydnc</v>
@@ -7455,7 +7476,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.999784860935</v>
-    <v>259</v>
+    <v>260</v>
     <v>5.7750000000000004</v>
     <v>11108900000</v>
     <v>AURORA INNOVATION, INC.</v>
@@ -7473,7 +7494,7 @@
     <v>2021</v>
   </rv>
   <rv s="2">
-    <v>260</v>
+    <v>261</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1p4kr&amp;q=XNYS%3aCACI&amp;form=skydnc</v>
@@ -7509,7 +7530,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.958333367969</v>
-    <v>262</v>
+    <v>263</v>
     <v>479.91</v>
     <v>10689250000</v>
     <v>CACI INTERNATIONAL INC.</v>
@@ -7527,7 +7548,7 @@
     <v>1985</v>
   </rv>
   <rv s="2">
-    <v>263</v>
+    <v>264</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1s2fr&amp;q=XNYS%3aEPAM&amp;form=skydnc</v>
@@ -7563,7 +7584,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.961634235937</v>
-    <v>265</v>
+    <v>266</v>
     <v>166.8279</v>
     <v>9744174404</v>
     <v>EPAM SYSTEMS, INC.</v>
@@ -7581,7 +7602,7 @@
     <v>2002</v>
   </rv>
   <rv s="2">
-    <v>266</v>
+    <v>267</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=bpwo9c&amp;q=XNYS%3aPSN&amp;form=skydnc</v>
@@ -7617,7 +7638,7 @@
     <v>Aerospace &amp; Defense</v>
     <v>Stock</v>
     <v>45891.999801353908</v>
-    <v>268</v>
+    <v>269</v>
     <v>78.33</v>
     <v>8524284000</v>
     <v>PARSONS CORPORATION</v>
@@ -7635,7 +7656,7 @@
     <v>1978</v>
   </rv>
   <rv s="2">
-    <v>269</v>
+    <v>270</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1tlpr&amp;q=XNYS%3aG&amp;form=skydnc</v>
@@ -7671,7 +7692,7 @@
     <v>Professional &amp; Commercial Services</v>
     <v>Stock</v>
     <v>45891.958333356248</v>
-    <v>271</v>
+    <v>272</v>
     <v>44.35</v>
     <v>7896178231</v>
     <v>GENPACT LIMITED</v>
@@ -7689,7 +7710,7 @@
     <v>2007</v>
   </rv>
   <rv s="2">
-    <v>272</v>
+    <v>273</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=c3twf2&amp;q=XNYS%3aKD&amp;form=skydnc</v>
@@ -7725,7 +7746,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.993314687497</v>
-    <v>274</v>
+    <v>275</v>
     <v>30.44</v>
     <v>7211692000</v>
     <v>KYNDRYL HOLDINGS, INC.</v>
@@ -7743,7 +7764,7 @@
     <v>2020</v>
   </rv>
   <rv s="2">
-    <v>275</v>
+    <v>276</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1si77&amp;q=XNAS%3aEXLS&amp;form=skydnc</v>
@@ -7779,7 +7800,7 @@
     <v>Professional &amp; Commercial Services</v>
     <v>Stock</v>
     <v>45891.89266045078</v>
-    <v>277</v>
+    <v>278</v>
     <v>43.73</v>
     <v>7114654000</v>
     <v>EXLSERVICE HOLDINGS, INC.</v>
@@ -7797,7 +7818,7 @@
     <v>2002</v>
   </rv>
   <rv s="2">
-    <v>278</v>
+    <v>279</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1tqdm&amp;q=XNAS%3aGDS&amp;form=skydnc</v>
@@ -7833,7 +7854,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.999506423439</v>
-    <v>280</v>
+    <v>281</v>
     <v>31.73</v>
     <v>6086963000</v>
     <v>GDS HOLDINGS LIMITED</v>
@@ -7851,7 +7872,7 @@
     <v>2006</v>
   </rv>
   <rv s="2">
-    <v>281</v>
+    <v>282</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a22gc7&amp;q=XNYS%3aSAIC&amp;form=skydnc</v>
@@ -7887,7 +7908,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.998901064064</v>
-    <v>283</v>
+    <v>284</v>
     <v>117.47</v>
     <v>5586769032</v>
     <v>SCIENCE APPLICATIONS INTERNATIONAL CORPORATION</v>
@@ -7905,7 +7926,7 @@
     <v>2013</v>
   </rv>
   <rv s="2">
-    <v>284</v>
+    <v>285</v>
   </rv>
   <rv s="7">
     <v>en-AE</v>
@@ -7954,7 +7975,7 @@
     <v>2016</v>
   </rv>
   <rv s="2">
-    <v>286</v>
+    <v>287</v>
   </rv>
   <rv s="7">
     <v>en-AE</v>
@@ -8003,7 +8024,7 @@
     <v>2020</v>
   </rv>
   <rv s="2">
-    <v>288</v>
+    <v>289</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a285oc&amp;q=XNAS%3aAPLD&amp;form=skydnc</v>
@@ -8039,7 +8060,7 @@
     <v>Financial Technology (Fintech) &amp; Infrastructure</v>
     <v>Stock</v>
     <v>45891.999782314066</v>
-    <v>290</v>
+    <v>291</v>
     <v>15.33</v>
     <v>4197392790</v>
     <v>APPLIED DIGITAL CORPORATION</v>
@@ -8057,7 +8078,7 @@
     <v>2001</v>
   </rv>
   <rv s="2">
-    <v>291</v>
+    <v>292</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1u8u2&amp;q=XNAS%3aVRRM&amp;form=skydnc</v>
@@ -8093,7 +8114,7 @@
     <v>Professional &amp; Commercial Services</v>
     <v>Stock</v>
     <v>45891.941470832811</v>
-    <v>293</v>
+    <v>294</v>
     <v>24.614999999999998</v>
     <v>4074672032</v>
     <v>VERRA MOBILITY CORPORATION</v>
@@ -8111,7 +8132,7 @@
     <v>2016</v>
   </rv>
   <rv s="2">
-    <v>294</v>
+    <v>295</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=bwtkar&amp;q=XNAS%3aCNXC&amp;form=skydnc</v>
@@ -8147,7 +8168,7 @@
     <v>Professional &amp; Commercial Services</v>
     <v>Stock</v>
     <v>45891.944591608597</v>
-    <v>296</v>
+    <v>297</v>
     <v>50.06</v>
     <v>3281718000</v>
     <v>CONCENTRIX CORPORATION</v>
@@ -8165,7 +8186,7 @@
     <v>2009</v>
   </rv>
   <rv s="2">
-    <v>297</v>
+    <v>298</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a25ylh&amp;q=XNYS%3aWNS&amp;form=skydnc</v>
@@ -8201,7 +8222,7 @@
     <v>Professional &amp; Commercial Services</v>
     <v>Stock</v>
     <v>45891.958333356248</v>
-    <v>299</v>
+    <v>300</v>
     <v>75.27</v>
     <v>3233342935</v>
     <v>WNS (HOLDINGS) LIMITED</v>
@@ -8219,7 +8240,7 @@
     <v>2002</v>
   </rv>
   <rv s="2">
-    <v>300</v>
+    <v>301</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1txbh&amp;q=XNYS%3aGLOB&amp;form=skydnc</v>
@@ -8255,13 +8276,13 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.995950775003</v>
-    <v>302</v>
+    <v>303</v>
     <v>67.13</v>
     <v>3080106000</v>
     <v>Globant SA</v>
     <v>Globant SA</v>
     <v>67.61</v>
-    <v>27.743400000000001</v>
+    <v>26.7714</v>
     <v>67.48</v>
     <v>69.930000000000007</v>
     <v>69.900000000000006</v>
@@ -8273,7 +8294,7 @@
     <v>2012</v>
   </rv>
   <rv s="2">
-    <v>303</v>
+    <v>304</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1pbww&amp;q=XNYS%3aCLVT&amp;form=skydnc</v>
@@ -8309,7 +8330,7 @@
     <v>Professional &amp; Commercial Services</v>
     <v>Stock</v>
     <v>45891.996912071096</v>
-    <v>305</v>
+    <v>306</v>
     <v>4.38</v>
     <v>3024900000</v>
     <v>CLARIVATE Plc</v>
@@ -8326,7 +8347,7 @@
     <v>2019</v>
   </rv>
   <rv s="2">
-    <v>306</v>
+    <v>307</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1rgur&amp;q=XNYS%3aDXC&amp;form=skydnc</v>
@@ -8362,7 +8383,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.958333356248</v>
-    <v>308</v>
+    <v>309</v>
     <v>13.765000000000001</v>
     <v>2550731475</v>
     <v>DXC TECHNOLOGY COMPANY</v>
@@ -8380,7 +8401,7 @@
     <v>2017</v>
   </rv>
   <rv s="2">
-    <v>309</v>
+    <v>310</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1nsxm&amp;q=XNYS%3aASGN&amp;form=skydnc</v>
@@ -8416,13 +8437,13 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.958471735939</v>
-    <v>311</v>
+    <v>312</v>
     <v>51.61</v>
     <v>2371332000</v>
     <v>ASGN Incorporated</v>
     <v>ASGN Incorporated</v>
     <v>52</v>
-    <v>17.2607</v>
+    <v>16.399899999999999</v>
     <v>51.44</v>
     <v>54.14</v>
     <v>54.14</v>
@@ -8434,7 +8455,7 @@
     <v>1992</v>
   </rv>
   <rv s="2">
-    <v>312</v>
+    <v>313</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a25fw7&amp;q=XNAS%3aVNET&amp;form=skydnc</v>
@@ -8470,7 +8491,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.988689409372</v>
-    <v>314</v>
+    <v>315</v>
     <v>7.4050000000000002</v>
     <v>2230224711</v>
     <v>VNET Group, Inc.</v>
@@ -8488,7 +8509,7 @@
     <v>2009</v>
   </rv>
   <rv s="2">
-    <v>315</v>
+    <v>316</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=c4efww&amp;q=XNYS%3aBBAI&amp;form=skydnc</v>
@@ -8524,7 +8545,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.999947094533</v>
-    <v>317</v>
+    <v>318</v>
     <v>5.26</v>
     <v>2038868000</v>
     <v>BigBear.ai Holdings, Inc.</v>
@@ -8541,7 +8562,7 @@
     <v>2020</v>
   </rv>
   <rv s="2">
-    <v>318</v>
+    <v>319</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1t92w&amp;q=XNAS%3aFORTY&amp;form=skydnc</v>
@@ -8577,7 +8598,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.840328818747</v>
-    <v>320</v>
+    <v>321</v>
     <v>128.7088</v>
     <v>1939607000</v>
     <v>FORMULA SYSTEMS (1985) LTD</v>
@@ -8595,7 +8616,7 @@
     <v>1985</v>
   </rv>
   <rv s="2">
-    <v>321</v>
+    <v>322</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1ycu2&amp;q=XNYS%3aNCR&amp;form=skydnc</v>
@@ -8631,7 +8652,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.958333344533</v>
-    <v>323</v>
+    <v>324</v>
     <v>12.91</v>
     <v>1896575000</v>
     <v>NCR VOYIX CORPORATION</v>
@@ -8648,7 +8669,7 @@
     <v>1926</v>
   </rv>
   <rv s="2">
-    <v>324</v>
+    <v>325</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=c1tlr7&amp;q=XNAS%3aTASK&amp;form=skydnc</v>
@@ -8684,7 +8705,7 @@
     <v>Professional &amp; Commercial Services</v>
     <v>Stock</v>
     <v>45891.840330381252</v>
-    <v>326</v>
+    <v>327</v>
     <v>17.25</v>
     <v>1562044532</v>
     <v>TASKUS, INC.</v>
@@ -8702,7 +8723,7 @@
     <v>2018</v>
   </rv>
   <rv s="2">
-    <v>327</v>
+    <v>328</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=c2pclh&amp;q=XNYS%3aNABL&amp;form=skydnc</v>
@@ -8738,7 +8759,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.958333344533</v>
-    <v>329</v>
+    <v>330</v>
     <v>7.6501000000000001</v>
     <v>1493027000</v>
     <v>N-ABLE, INC.</v>
@@ -8756,7 +8777,7 @@
     <v>2020</v>
   </rv>
   <rv s="2">
-    <v>330</v>
+    <v>331</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a22ugh&amp;q=XNAS%3aSGH&amp;form=skydnc</v>
@@ -8792,7 +8813,7 @@
     <v>Semiconductors &amp; Semiconductor Equipment</v>
     <v>Stock</v>
     <v>45891.994189664059</v>
-    <v>332</v>
+    <v>333</v>
     <v>23.25</v>
     <v>1275967028</v>
     <v>PENGUIN SOLUTIONS, INC.</v>
@@ -8810,7 +8831,7 @@
     <v>2025</v>
   </rv>
   <rv s="2">
-    <v>333</v>
+    <v>334</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1vla2&amp;q=XNAS%3aINOD&amp;form=skydnc</v>
@@ -8846,7 +8867,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.999687985939</v>
-    <v>335</v>
+    <v>336</v>
     <v>36.840000000000003</v>
     <v>1225420000</v>
     <v>INNODATA INC.</v>
@@ -8864,7 +8885,7 @@
     <v>1988</v>
   </rv>
   <rv s="2">
-    <v>336</v>
+    <v>337</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1xk9c&amp;q=XNAS%3aMGIC&amp;form=skydnc</v>
@@ -8900,7 +8921,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.836206296095</v>
-    <v>338</v>
+    <v>339</v>
     <v>19.79</v>
     <v>3279900000</v>
     <v>MAGIC SOFTWARE ENTERPRISES LTD.</v>
@@ -8918,7 +8939,7 @@
     <v>1983</v>
   </rv>
   <rv s="2">
-    <v>339</v>
+    <v>340</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=bnmncw&amp;q=XNAS%3aGDYN&amp;form=skydnc</v>
@@ -8954,7 +8975,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.867416828129</v>
-    <v>341</v>
+    <v>342</v>
     <v>7.99</v>
     <v>685826700</v>
     <v>GRID DYNAMICS HOLDINGS, INC.</v>
@@ -8972,7 +8993,7 @@
     <v>2018</v>
   </rv>
   <rv s="2">
-    <v>342</v>
+    <v>343</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1uibh&amp;q=XNAS%3aHCKT&amp;form=skydnc</v>
@@ -9008,7 +9029,7 @@
     <v>Professional &amp; Commercial Services</v>
     <v>Stock</v>
     <v>45891.90644701328</v>
-    <v>344</v>
+    <v>345</v>
     <v>20.170000000000002</v>
     <v>580200452</v>
     <v>THE HACKETT GROUP, INC.</v>
@@ -9026,7 +9047,7 @@
     <v>1997</v>
   </rv>
   <rv s="2">
-    <v>345</v>
+    <v>346</v>
   </rv>
   <rv s="11">
     <v>en-AE</v>
@@ -9074,7 +9095,7 @@
     <v>2022</v>
   </rv>
   <rv s="2">
-    <v>347</v>
+    <v>348</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a26arw&amp;q=XNAS%3aXRX&amp;form=skydnc</v>
@@ -9110,7 +9131,7 @@
     <v>Office Equipment</v>
     <v>Stock</v>
     <v>45891.999659003908</v>
-    <v>349</v>
+    <v>350</v>
     <v>3.7</v>
     <v>484443190</v>
     <v>Xerox Holdings Corp</v>
@@ -9128,7 +9149,7 @@
     <v>2019</v>
   </rv>
   <rv s="2">
-    <v>350</v>
+    <v>351</v>
   </rv>
   <rv s="7">
     <v>en-AE</v>
@@ -9177,7 +9198,7 @@
     <v>2024</v>
   </rv>
   <rv s="2">
-    <v>352</v>
+    <v>353</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1pzu2&amp;q=XNAS%3aCNDT&amp;form=skydnc</v>
@@ -9213,7 +9234,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.996829628908</v>
-    <v>354</v>
+    <v>355</v>
     <v>2.5499999999999998</v>
     <v>442327300</v>
     <v>CONDUENT INCORPORATED</v>
@@ -9231,7 +9252,7 @@
     <v>2016</v>
   </rv>
   <rv s="2">
-    <v>355</v>
+    <v>356</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a2z4lh&amp;q=OTCM%3aTSSI&amp;form=skydnc</v>
@@ -9267,7 +9288,7 @@
     <v>Professional &amp; Commercial Services</v>
     <v>Stock</v>
     <v>45891.998960971876</v>
-    <v>357</v>
+    <v>358</v>
     <v>14.37</v>
     <v>418726400</v>
     <v>TSS, INC.</v>
@@ -9285,7 +9306,7 @@
     <v>2004</v>
   </rv>
   <rv s="2">
-    <v>358</v>
+    <v>359</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=azgvgh&amp;q=XNAS%3aIBEX&amp;form=skydnc</v>
@@ -9321,7 +9342,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.840329108592</v>
-    <v>360</v>
+    <v>361</v>
     <v>29.27</v>
     <v>404114000</v>
     <v>IBEX Limited</v>
@@ -9339,7 +9360,7 @@
     <v>2017</v>
   </rv>
   <rv s="2">
-    <v>361</v>
+    <v>362</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1w88m&amp;q=XNAS%3aMFH&amp;form=skydnc</v>
@@ -9375,7 +9396,7 @@
     <v>Financial Technology (Fintech) &amp; Infrastructure</v>
     <v>Stock</v>
     <v>45891.996535057813</v>
-    <v>363</v>
+    <v>364</v>
     <v>4.4000000000000004</v>
     <v>314611606</v>
     <v>Mercurity Fintech Holding Inc</v>
@@ -9393,7 +9414,7 @@
     <v>2011</v>
   </rv>
   <rv s="2">
-    <v>364</v>
+    <v>365</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a24vh7&amp;q=XNYS%3aUIS&amp;form=skydnc</v>
@@ -9429,7 +9450,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.958333333336</v>
-    <v>366</v>
+    <v>367</v>
     <v>3.8650000000000002</v>
     <v>298717800</v>
     <v>UNISYS CORPORATION</v>
@@ -9446,7 +9467,7 @@
     <v>1984</v>
   </rv>
   <rv s="2">
-    <v>367</v>
+    <v>368</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1vfpr&amp;q=XNAS%3aIII&amp;form=skydnc</v>
@@ -9482,7 +9503,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.97635643516</v>
-    <v>369</v>
+    <v>370</v>
     <v>4.82</v>
     <v>242423200</v>
     <v>INFORMATION SERVICES GROUP, INC.</v>
@@ -9500,7 +9521,7 @@
     <v>2006</v>
   </rv>
   <rv s="2">
-    <v>370</v>
+    <v>371</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a24lim&amp;q=XNAS%3aTTEC&amp;form=skydnc</v>
@@ -9536,7 +9557,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.921280103903</v>
-    <v>372</v>
+    <v>373</v>
     <v>3.64</v>
     <v>184161300</v>
     <v>TTEC Holdings, Inc.</v>
@@ -9554,7 +9575,7 @@
     <v>1994</v>
   </rv>
   <rv s="2">
-    <v>373</v>
+    <v>374</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1qfar&amp;q=XNAS%3aCSPI&amp;form=skydnc</v>
@@ -9590,7 +9611,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.840325034376</v>
-    <v>375</v>
+    <v>376</v>
     <v>11.81</v>
     <v>125633344</v>
     <v>CSP, INC.</v>
@@ -9608,7 +9629,7 @@
     <v>1968</v>
   </rv>
   <rv s="2">
-    <v>376</v>
+    <v>377</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a2r56h&amp;q=OTCM%3aONOV&amp;form=skydnc</v>
@@ -9644,7 +9665,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.99677905078</v>
-    <v>378</v>
+    <v>379</v>
     <v>0.98</v>
     <v>95790600</v>
     <v>CASTELLUM, INC.</v>
@@ -9661,7 +9682,7 @@
     <v>2010</v>
   </rv>
   <rv s="2">
-    <v>379</v>
+    <v>380</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=bwxx4c&amp;q=XNAS%3aDSAC&amp;form=skydnc</v>
@@ -9697,7 +9718,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.997715057812</v>
-    <v>381</v>
+    <v>382</v>
     <v>0.50019999999999998</v>
     <v>88562460</v>
     <v>FISCALNOTE HOLDINGS, INC.</v>
@@ -9714,7 +9735,7 @@
     <v>2022</v>
   </rv>
   <rv s="2">
-    <v>382</v>
+    <v>383</v>
   </rv>
   <rv s="11">
     <v>en-AE</v>
@@ -9762,7 +9783,7 @@
     <v>2021</v>
   </rv>
   <rv s="2">
-    <v>384</v>
+    <v>385</v>
   </rv>
   <rv s="11">
     <v>en-AE</v>
@@ -9779,9 +9800,9 @@
     <v>4.74</v>
     <v>0.17199999999999999</v>
     <v>-5.7099999999999998E-2</v>
-    <v>4.7355000000000001E-2</v>
+    <v>2.7456000000000001E-2</v>
     <v>-6.7089999999999997E-2</v>
-    <v>3.7600000000000001E-2</v>
+    <v>2.18E-2</v>
     <v>USD</v>
     <v>Trident Digital Tech Holdings Ltd is a Singapore-based company, which provides digital transformation in digital optimization, technology services, and Web 3.0 activation worldwide. The Company offers commercial and technological digital solutions designed to optimize its clients’ experience with their end-users by promoting digital adoption and self-service. Tridentity, the Company’s flagship product, is a blockchain-based identity solution designed to provide secure single sign-on authentication capabilities to integrated third-party systems across various industries. Tridentity offers unparalleled security features, ensuring the protection of sensitive information and preventing potential threats. Its solutions and services include business consulting and IT customization. It provides customized solutions and services that address the specific needs of clients in its vertical markets. Its primary vertical industries include e-commerce, food and beverage, wholesale, and retail.</v>
     <v>23</v>
@@ -9801,7 +9822,7 @@
     <v>0</v>
     <v>0.85109999999999997</v>
     <v>0.79400000000000004</v>
-    <v>0.83160000000000001</v>
+    <v>0.81579999999999997</v>
     <v>9615070</v>
     <v>TDTH</v>
     <v>Trident Digital Tech Holdings Ltd (XNAS:TDTH)</v>
@@ -9810,7 +9831,7 @@
     <v>2023</v>
   </rv>
   <rv s="2">
-    <v>386</v>
+    <v>387</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a25pp2&amp;q=XNYS%3aBTCM&amp;form=skydnc</v>
@@ -9846,7 +9867,7 @@
     <v>Financial Technology (Fintech) &amp; Infrastructure</v>
     <v>Stock</v>
     <v>45891.994920138284</v>
-    <v>388</v>
+    <v>389</v>
     <v>2.9550999999999998</v>
     <v>51308990</v>
     <v>BIT Mining Limited</v>
@@ -9863,7 +9884,7 @@
     <v>2007</v>
   </rv>
   <rv s="2">
-    <v>389</v>
+    <v>390</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a2658m&amp;q=XNYS%3aWYY&amp;form=skydnc</v>
@@ -9899,7 +9920,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.879628923438</v>
-    <v>391</v>
+    <v>392</v>
     <v>3.76</v>
     <v>41356310</v>
     <v>WIDEPOINT CORPORATION</v>
@@ -9916,7 +9937,7 @@
     <v>1997</v>
   </rv>
   <rv s="2">
-    <v>392</v>
+    <v>393</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a2et8m&amp;q=XNAS%3aDTST&amp;form=skydnc</v>
@@ -9952,7 +9973,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.996161435156</v>
-    <v>394</v>
+    <v>395</v>
     <v>4.5324999999999998</v>
     <v>33915580</v>
     <v>DATA STORAGE CORPORATION</v>
@@ -9970,7 +9991,7 @@
     <v>2007</v>
   </rv>
   <rv s="2">
-    <v>395</v>
+    <v>396</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=c21ypr&amp;q=XNAS%3aPLMI&amp;form=skydnc</v>
@@ -10006,7 +10027,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.999780960155</v>
-    <v>397</v>
+    <v>398</v>
     <v>0.56100000000000005</v>
     <v>30606540</v>
     <v>VEEA, INC.</v>
@@ -10024,7 +10045,7 @@
     <v>2024</v>
   </rv>
   <rv s="2">
-    <v>398</v>
+    <v>399</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=b12pa2&amp;q=XNAS%3aCLPS&amp;form=skydnc</v>
@@ -10060,7 +10081,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.840328228907</v>
-    <v>400</v>
+    <v>401</v>
     <v>1.0058</v>
     <v>28266100</v>
     <v>CLPS Incorporation</v>
@@ -10078,7 +10099,7 @@
     <v>2017</v>
   </rv>
   <rv s="2">
-    <v>401</v>
+    <v>402</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=br8z2w&amp;q=XNAS%3aJFU&amp;form=skydnc</v>
@@ -10114,7 +10135,7 @@
     <v>Financial Technology (Fintech) &amp; Infrastructure</v>
     <v>Stock</v>
     <v>45891.995879560156</v>
-    <v>403</v>
+    <v>404</v>
     <v>2</v>
     <v>17168970</v>
     <v>9F Inc</v>
@@ -10132,7 +10153,7 @@
     <v>2014</v>
   </rv>
   <rv s="2">
-    <v>404</v>
+    <v>405</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=c5uoyc&amp;q=XNAS%3aWAVS&amp;form=skydnc</v>
@@ -10168,7 +10189,7 @@
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
     <v>45891.999969745309</v>
-    <v>406</v>
+    <v>407</v>
     <v>0.31109999999999999</v>
     <v>16353480</v>
     <v>CYCURION, INC.</v>
@@ -10186,7 +10207,7 @@
     <v>2021</v>
   </rv>
   <rv s="2">
-    <v>407</v>
+    <v>408</v>
   </rv>
   <rv s="11">
     <v>en-AE</v>
@@ -10234,7 +10255,7 @@
     <v>2021</v>
   </rv>
   <rv s="2">
-    <v>409</v>
+    <v>410</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=c2ikdm&amp;q=XNAS%3aSAI&amp;form=skydnc</v>
@@ -10270,7 +10291,7 @@
     <v>Computers, Phones &amp; Household Electronics</v>
     <v>Stock</v>
     <v>45891.906913680468</v>
-    <v>411</v>
+    <v>412</v>
     <v>7.01</v>
     <v>12796535</v>
     <v>SAIHEAT Limited</v>
@@ -10288,7 +10309,7 @@
     <v>2021</v>
   </rv>
   <rv s="2">
-    <v>412</v>
+    <v>413</v>
   </rv>
   <rv s="7">
     <v>en-AE</v>
@@ -10337,7 +10358,7 @@
     <v>2022</v>
   </rv>
   <rv s="2">
-    <v>414</v>
+    <v>415</v>
   </rv>
   <rv s="11">
     <v>en-AE</v>
@@ -10385,7 +10406,7 @@
     <v>2023</v>
   </rv>
   <rv s="2">
-    <v>416</v>
+    <v>417</v>
   </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=c6qqz2&amp;q=XNAS%3aJZ&amp;form=skydnc</v>
@@ -10420,7 +10441,7 @@
     <v>Professional &amp; Business Education</v>
     <v>Stock</v>
     <v>45891.864357500002</v>
-    <v>418</v>
+    <v>419</v>
     <v>1.6</v>
     <v>4509600</v>
     <v>Jianzhi Education Technology Group Co Ltd</v>
@@ -10438,7 +10459,7 @@
     <v>2018</v>
   </rv>
   <rv s="2">
-    <v>419</v>
+    <v>420</v>
   </rv>
 </rvData>
 </file>
@@ -12237,7 +12258,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C73BEF28-9B3D-415B-9025-F87DF0281B83}">
-  <dimension ref="B1:K77"/>
+  <dimension ref="B1:L77"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="46.44140625" customWidth="1"/>
@@ -12249,9 +12270,10 @@
     <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="17.5546875" customWidth="1"/>
     <col min="11" max="11" width="27.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C1" s="18" t="s">
         <v>154</v>
       </c>
@@ -12279,8 +12301,11 @@
       <c r="K1" s="19" t="s">
         <v>306</v>
       </c>
+      <c r="L1" s="34" t="s">
+        <v>307</v>
+      </c>
     </row>
-    <row r="2" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C2" s="20" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
@@ -12309,8 +12334,12 @@
         <f t="array" aca="1" ref="K2" ca="1">_FV(C2,"Shares outstanding",TRUE)</f>
         <v>1060439000</v>
       </c>
+      <c r="L2" t="str" cm="1">
+        <f t="array" aca="1" ref="L2" ca="1">_FV(C2,"Ticker symbol",TRUE)</f>
+        <v>GE</v>
+      </c>
     </row>
-    <row r="3" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C3" s="26" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
@@ -12339,8 +12368,12 @@
         <f t="array" aca="1" ref="K3" ca="1">_FV(C3,"Shares outstanding",TRUE)</f>
         <v>1338542000</v>
       </c>
+      <c r="L3" t="str" cm="1">
+        <f t="array" aca="1" ref="L3" ca="1">_FV(C3,"Ticker symbol",TRUE)</f>
+        <v>RTX</v>
+      </c>
     </row>
-    <row r="4" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C4" s="20" t="e" vm="3">
         <v>#VALUE!</v>
       </c>
@@ -12369,8 +12402,12 @@
         <f t="array" aca="1" ref="K4" ca="1">_FV(C4,"Shares outstanding",TRUE)</f>
         <v>756157700</v>
       </c>
+      <c r="L4" t="str" cm="1">
+        <f t="array" aca="1" ref="L4" ca="1">_FV(C4,"Ticker symbol",TRUE)</f>
+        <v>BA</v>
+      </c>
     </row>
-    <row r="5" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C5" s="26" t="e" vm="4">
         <v>#VALUE!</v>
       </c>
@@ -12399,8 +12436,12 @@
         <f t="array" aca="1" ref="K5" ca="1">_FV(C5,"Shares outstanding",TRUE)</f>
         <v>233465100</v>
       </c>
+      <c r="L5" t="str" cm="1">
+        <f t="array" aca="1" ref="L5" ca="1">_FV(C5,"Ticker symbol",TRUE)</f>
+        <v>LMT</v>
+      </c>
     </row>
-    <row r="6" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C6" s="20" t="e" vm="5">
         <v>#VALUE!</v>
       </c>
@@ -12429,8 +12470,12 @@
         <f t="array" aca="1" ref="K6" ca="1">_FV(C6,"Shares outstanding",TRUE)</f>
         <v>268993300</v>
       </c>
+      <c r="L6" t="str" cm="1">
+        <f t="array" aca="1" ref="L6" ca="1">_FV(C6,"Ticker symbol",TRUE)</f>
+        <v>GD</v>
+      </c>
     </row>
-    <row r="7" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C7" s="26" t="e" vm="6">
         <v>#VALUE!</v>
       </c>
@@ -12459,8 +12504,12 @@
         <f t="array" aca="1" ref="K7" ca="1">_FV(C7,"Shares outstanding",TRUE)</f>
         <v>143183000</v>
       </c>
+      <c r="L7" t="str" cm="1">
+        <f t="array" aca="1" ref="L7" ca="1">_FV(C7,"Ticker symbol",TRUE)</f>
+        <v>NOC</v>
+      </c>
     </row>
-    <row r="8" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C8" s="20" t="e" vm="7">
         <v>#VALUE!</v>
       </c>
@@ -12489,8 +12538,12 @@
         <f t="array" aca="1" ref="K8" ca="1">_FV(C8,"Shares outstanding",TRUE)</f>
         <v>56350280</v>
       </c>
+      <c r="L8" t="str" cm="1">
+        <f t="array" aca="1" ref="L8" ca="1">_FV(C8,"Ticker symbol",TRUE)</f>
+        <v>TDG</v>
+      </c>
     </row>
-    <row r="9" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C9" s="26" t="e" vm="8">
         <v>#VALUE!</v>
       </c>
@@ -12519,8 +12572,12 @@
         <f t="array" aca="1" ref="K9" ca="1">_FV(C9,"Shares outstanding",TRUE)</f>
         <v>403126300</v>
       </c>
+      <c r="L9" t="str" cm="1">
+        <f t="array" aca="1" ref="L9" ca="1">_FV(C9,"Ticker symbol",TRUE)</f>
+        <v>HWM</v>
+      </c>
     </row>
-    <row r="10" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C10" s="20" t="e" vm="9">
         <v>#VALUE!</v>
       </c>
@@ -12549,8 +12606,12 @@
         <f t="array" aca="1" ref="K10" ca="1">_FV(C10,"Shares outstanding",TRUE)</f>
         <v>78504440</v>
       </c>
+      <c r="L10" t="str" cm="1">
+        <f t="array" aca="1" ref="L10" ca="1">_FV(C10,"Ticker symbol",TRUE)</f>
+        <v>AXON</v>
+      </c>
     </row>
-    <row r="11" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C11" s="26" t="e" vm="10">
         <v>#VALUE!</v>
       </c>
@@ -12579,8 +12640,12 @@
         <f t="array" aca="1" ref="K11" ca="1">_FV(C11,"Shares outstanding",TRUE)</f>
         <v>187094800</v>
       </c>
+      <c r="L11" t="str" cm="1">
+        <f t="array" aca="1" ref="L11" ca="1">_FV(C11,"Ticker symbol",TRUE)</f>
+        <v>LHX</v>
+      </c>
     </row>
-    <row r="12" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C12" s="20" t="e" vm="11">
         <v>#VALUE!</v>
       </c>
@@ -12609,8 +12674,12 @@
         <f t="array" aca="1" ref="K12" ca="1">_FV(C12,"Shares outstanding",TRUE)</f>
         <v>139104100</v>
       </c>
+      <c r="L12" t="str" cm="1">
+        <f t="array" aca="1" ref="L12" ca="1">_FV(C12,"Ticker symbol",TRUE)</f>
+        <v>HEI</v>
+      </c>
     </row>
-    <row r="13" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C13" s="26" t="e" vm="12">
         <v>#VALUE!</v>
       </c>
@@ -12639,8 +12708,12 @@
         <f t="array" aca="1" ref="K13" ca="1">_FV(C13,"Shares outstanding",TRUE)</f>
         <v>139104100</v>
       </c>
+      <c r="L13" t="str" cm="1">
+        <f t="array" aca="1" ref="L13" ca="1">_FV(C13,"Ticker symbol",TRUE)</f>
+        <v>HEI.A</v>
+      </c>
     </row>
-    <row r="14" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C14" s="20" t="e" vm="13">
         <v>#VALUE!</v>
       </c>
@@ -12669,8 +12742,12 @@
         <f t="array" aca="1" ref="K14" ca="1">_FV(C14,"Shares outstanding",TRUE)</f>
         <v>482413300</v>
       </c>
+      <c r="L14" t="str" cm="1">
+        <f t="array" aca="1" ref="L14" ca="1">_FV(C14,"Ticker symbol",TRUE)</f>
+        <v>RKLB</v>
+      </c>
     </row>
-    <row r="15" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C15" s="26" t="e" vm="14">
         <v>#VALUE!</v>
       </c>
@@ -12699,8 +12776,12 @@
         <f t="array" aca="1" ref="K15" ca="1">_FV(C15,"Shares outstanding",TRUE)</f>
         <v>46346340</v>
       </c>
+      <c r="L15" t="str" cm="1">
+        <f t="array" aca="1" ref="L15" ca="1">_FV(C15,"Ticker symbol",TRUE)</f>
+        <v>ESLT</v>
+      </c>
     </row>
-    <row r="16" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C16" s="20" t="e" vm="15">
         <v>#VALUE!</v>
       </c>
@@ -12729,8 +12810,12 @@
         <f t="array" aca="1" ref="K16" ca="1">_FV(C16,"Shares outstanding",TRUE)</f>
         <v>37678110</v>
       </c>
+      <c r="L16" t="str" cm="1">
+        <f t="array" aca="1" ref="L16" ca="1">_FV(C16,"Ticker symbol",TRUE)</f>
+        <v>CW</v>
+      </c>
     </row>
-    <row r="17" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C17" s="26" t="e" vm="16">
         <v>#VALUE!</v>
       </c>
@@ -12759,8 +12844,12 @@
         <f t="array" aca="1" ref="K17" ca="1">_FV(C17,"Shares outstanding",TRUE)</f>
         <v>91398740</v>
       </c>
+      <c r="L17" t="str" cm="1">
+        <f t="array" aca="1" ref="L17" ca="1">_FV(C17,"Ticker symbol",TRUE)</f>
+        <v>BWXT</v>
+      </c>
     </row>
-    <row r="18" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C18" s="20" t="e" vm="17">
         <v>#VALUE!</v>
       </c>
@@ -12789,8 +12878,12 @@
         <f t="array" aca="1" ref="K18" ca="1">_FV(C18,"Shares outstanding",TRUE)</f>
         <v>59966220</v>
       </c>
+      <c r="L18" t="str" cm="1">
+        <f t="array" aca="1" ref="L18" ca="1">_FV(C18,"Ticker symbol",TRUE)</f>
+        <v>WWD</v>
+      </c>
     </row>
-    <row r="19" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C19" s="26" t="e" vm="18">
         <v>#VALUE!</v>
       </c>
@@ -12819,8 +12912,12 @@
         <f t="array" aca="1" ref="K19" ca="1">_FV(C19,"Shares outstanding",TRUE)</f>
         <v>178205300</v>
       </c>
+      <c r="L19" t="str" cm="1">
+        <f t="array" aca="1" ref="L19" ca="1">_FV(C19,"Ticker symbol",TRUE)</f>
+        <v>TXT</v>
+      </c>
     </row>
-    <row r="20" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C20" s="20" t="e" vm="19">
         <v>#VALUE!</v>
       </c>
@@ -12849,8 +12946,12 @@
         <f t="array" aca="1" ref="K20" ca="1">_FV(C20,"Shares outstanding",TRUE)</f>
         <v>49932230</v>
       </c>
+      <c r="L20" t="str" cm="1">
+        <f t="array" aca="1" ref="L20" ca="1">_FV(C20,"Ticker symbol",TRUE)</f>
+        <v>AVAV</v>
+      </c>
     </row>
-    <row r="21" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C21" s="26" t="e" vm="20">
         <v>#VALUE!</v>
       </c>
@@ -12879,8 +12980,12 @@
         <f t="array" aca="1" ref="K21" ca="1">_FV(C21,"Shares outstanding",TRUE)</f>
         <v>168794500</v>
       </c>
+      <c r="L21" t="str" cm="1">
+        <f t="array" aca="1" ref="L21" ca="1">_FV(C21,"Ticker symbol",TRUE)</f>
+        <v>KTOS</v>
+      </c>
     </row>
-    <row r="22" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C22" s="20" t="e" vm="21">
         <v>#VALUE!</v>
       </c>
@@ -12909,8 +13014,12 @@
         <f t="array" aca="1" ref="K22" ca="1">_FV(C22,"Shares outstanding",TRUE)</f>
         <v>266123600</v>
       </c>
+      <c r="L22" t="str" cm="1">
+        <f t="array" aca="1" ref="L22" ca="1">_FV(C22,"Ticker symbol",TRUE)</f>
+        <v>DRS</v>
+      </c>
     </row>
-    <row r="23" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C23" s="26" t="e" vm="22">
         <v>#VALUE!</v>
       </c>
@@ -12939,8 +13048,12 @@
         <f t="array" aca="1" ref="K23" ca="1">_FV(C23,"Shares outstanding",TRUE)</f>
         <v>39240630</v>
       </c>
+      <c r="L23" t="str" cm="1">
+        <f t="array" aca="1" ref="L23" ca="1">_FV(C23,"Ticker symbol",TRUE)</f>
+        <v>HII</v>
+      </c>
     </row>
-    <row r="24" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C24" s="20" t="e" vm="23">
         <v>#VALUE!</v>
       </c>
@@ -12969,8 +13082,12 @@
         <f t="array" aca="1" ref="K24" ca="1">_FV(C24,"Shares outstanding",TRUE)</f>
         <v>185116300</v>
       </c>
+      <c r="L24" t="str" cm="1">
+        <f t="array" aca="1" ref="L24" ca="1">_FV(C24,"Ticker symbol",TRUE)</f>
+        <v>ERJ</v>
+      </c>
     </row>
-    <row r="25" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C25" s="26" t="e" vm="24">
         <v>#VALUE!</v>
       </c>
@@ -12999,8 +13116,12 @@
         <f t="array" aca="1" ref="K25" ca="1">_FV(C25,"Shares outstanding",TRUE)</f>
         <v>334470200</v>
       </c>
+      <c r="L25" t="str" cm="1">
+        <f t="array" aca="1" ref="L25" ca="1">_FV(C25,"Ticker symbol",TRUE)</f>
+        <v>SARO</v>
+      </c>
     </row>
-    <row r="26" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C26" s="20" t="e" vm="25">
         <v>#VALUE!</v>
       </c>
@@ -13029,8 +13150,12 @@
         <f t="array" aca="1" ref="K26" ca="1">_FV(C26,"Shares outstanding",TRUE)</f>
         <v>320726200</v>
       </c>
+      <c r="L26" t="str" cm="1">
+        <f t="array" aca="1" ref="L26" ca="1">_FV(C26,"Ticker symbol",TRUE)</f>
+        <v>CAE</v>
+      </c>
     </row>
-    <row r="27" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="27" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C27" s="26" t="e" vm="26">
         <v>#VALUE!</v>
       </c>
@@ -13059,8 +13184,12 @@
         <f t="array" aca="1" ref="K27" ca="1">_FV(C27,"Shares outstanding",TRUE)</f>
         <v>132322400</v>
       </c>
+      <c r="L27" t="str" cm="1">
+        <f t="array" aca="1" ref="L27" ca="1">_FV(C27,"Ticker symbol",TRUE)</f>
+        <v>KRMN</v>
+      </c>
     </row>
-    <row r="28" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C28" s="20" t="e" vm="27">
         <v>#VALUE!</v>
       </c>
@@ -13089,8 +13218,12 @@
         <f t="array" aca="1" ref="K28" ca="1">_FV(C28,"Shares outstanding",TRUE)</f>
         <v>93622470</v>
       </c>
+      <c r="L28" t="str" cm="1">
+        <f t="array" aca="1" ref="L28" ca="1">_FV(C28,"Ticker symbol",TRUE)</f>
+        <v>LOAR</v>
+      </c>
     </row>
-    <row r="29" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="29" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C29" s="26" t="e" vm="28">
         <v>#VALUE!</v>
       </c>
@@ -13119,8 +13252,12 @@
         <f t="array" aca="1" ref="K29" ca="1">_FV(C29,"Shares outstanding",TRUE)</f>
         <v>43009880</v>
       </c>
+      <c r="L29" t="str" cm="1">
+        <f t="array" aca="1" ref="L29" ca="1">_FV(C29,"Ticker symbol",TRUE)</f>
+        <v>FLY</v>
+      </c>
     </row>
-    <row r="30" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="30" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C30" s="20" t="e" vm="29">
         <v>#VALUE!</v>
       </c>
@@ -13149,8 +13286,12 @@
         <f t="array" aca="1" ref="K30" ca="1">_FV(C30,"Shares outstanding",TRUE)</f>
         <v>31677810</v>
       </c>
+      <c r="L30" t="str" cm="1">
+        <f t="array" aca="1" ref="L30" ca="1">_FV(C30,"Ticker symbol",TRUE)</f>
+        <v>MOG.A</v>
+      </c>
     </row>
-    <row r="31" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="31" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C31" s="26" t="e" vm="30">
         <v>#VALUE!</v>
       </c>
@@ -13179,8 +13320,12 @@
         <f t="array" aca="1" ref="K31" ca="1">_FV(C31,"Shares outstanding",TRUE)</f>
         <v>31677810</v>
       </c>
+      <c r="L31" t="str" cm="1">
+        <f t="array" aca="1" ref="L31" ca="1">_FV(C31,"Ticker symbol",TRUE)</f>
+        <v>MOG.B</v>
+      </c>
     </row>
-    <row r="32" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="32" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C32" s="20" t="e" vm="31">
         <v>#VALUE!</v>
       </c>
@@ -13209,8 +13354,12 @@
         <f t="array" aca="1" ref="K32" ca="1">_FV(C32,"Shares outstanding",TRUE)</f>
         <v>645026300</v>
       </c>
+      <c r="L32" t="str" cm="1">
+        <f t="array" aca="1" ref="L32" ca="1">_FV(C32,"Ticker symbol",TRUE)</f>
+        <v>ACHR</v>
+      </c>
     </row>
-    <row r="33" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="33" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C33" s="26" t="e" vm="32">
         <v>#VALUE!</v>
       </c>
@@ -13239,8 +13388,12 @@
         <f t="array" aca="1" ref="K33" ca="1">_FV(C33,"Shares outstanding",TRUE)</f>
         <v>79563350</v>
       </c>
+      <c r="L33" t="str" cm="1">
+        <f t="array" aca="1" ref="L33" ca="1">_FV(C33,"Ticker symbol",TRUE)</f>
+        <v>HXL</v>
+      </c>
     </row>
-    <row r="34" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="34" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C34" s="20" t="e" vm="33">
         <v>#VALUE!</v>
       </c>
@@ -13269,8 +13422,12 @@
         <f t="array" aca="1" ref="K34" ca="1">_FV(C34,"Shares outstanding",TRUE)</f>
         <v>117419200</v>
       </c>
+      <c r="L34" t="str" cm="1">
+        <f t="array" aca="1" ref="L34" ca="1">_FV(C34,"Ticker symbol",TRUE)</f>
+        <v>SPR</v>
+      </c>
     </row>
-    <row r="35" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="35" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C35" s="26" t="e" vm="34">
         <v>#VALUE!</v>
       </c>
@@ -13299,8 +13456,12 @@
         <f t="array" aca="1" ref="K35" ca="1">_FV(C35,"Shares outstanding",TRUE)</f>
         <v>59915670</v>
       </c>
+      <c r="L35" t="str" cm="1">
+        <f t="array" aca="1" ref="L35" ca="1">_FV(C35,"Ticker symbol",TRUE)</f>
+        <v>MRCY</v>
+      </c>
     </row>
-    <row r="36" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="36" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C36" s="20" t="e" vm="35">
         <v>#VALUE!</v>
       </c>
@@ -13329,8 +13490,12 @@
         <f t="array" aca="1" ref="K36" ca="1">_FV(C36,"Shares outstanding",TRUE)</f>
         <v>20676320</v>
       </c>
+      <c r="L36" t="str" cm="1">
+        <f t="array" aca="1" ref="L36" ca="1">_FV(C36,"Ticker symbol",TRUE)</f>
+        <v>VSEC</v>
+      </c>
     </row>
-    <row r="37" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="37" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C37" s="26" t="e" vm="36">
         <v>#VALUE!</v>
       </c>
@@ -13359,8 +13524,12 @@
         <f t="array" aca="1" ref="K37" ca="1">_FV(C37,"Shares outstanding",TRUE)</f>
         <v>35964150</v>
       </c>
+      <c r="L37" t="str" cm="1">
+        <f t="array" aca="1" ref="L37" ca="1">_FV(C37,"Ticker symbol",TRUE)</f>
+        <v>AIR</v>
+      </c>
     </row>
-    <row r="38" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="38" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C38" s="20" t="e" vm="37">
         <v>#VALUE!</v>
       </c>
@@ -13389,8 +13558,12 @@
         <f t="array" aca="1" ref="K38" ca="1">_FV(C38,"Shares outstanding",TRUE)</f>
         <v>303430900</v>
       </c>
+      <c r="L38" t="str" cm="1">
+        <f t="array" aca="1" ref="L38" ca="1">_FV(C38,"Ticker symbol",TRUE)</f>
+        <v>PL</v>
+      </c>
     </row>
-    <row r="39" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="39" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C39" s="26" t="e" vm="38">
         <v>#VALUE!</v>
       </c>
@@ -13419,8 +13592,12 @@
         <f t="array" aca="1" ref="K39" ca="1">_FV(C39,"Shares outstanding",TRUE)</f>
         <v>31709820</v>
       </c>
+      <c r="L39" t="str" cm="1">
+        <f t="array" aca="1" ref="L39" ca="1">_FV(C39,"Ticker symbol",TRUE)</f>
+        <v>VVX</v>
+      </c>
     </row>
-    <row r="40" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="40" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C40" s="20" t="s">
         <v>75</v>
       </c>
@@ -13449,9 +13626,13 @@
         <f t="array" ref="K40">_FV(C40,"Shares outstanding",TRUE)</f>
         <v>#VALUE!</v>
       </c>
+      <c r="L40" t="e" cm="1" vm="40">
+        <f t="array" ref="L40">_FV(C40,"Ticker symbol",TRUE)</f>
+        <v>#VALUE!</v>
+      </c>
     </row>
-    <row r="41" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C41" s="26" t="e" vm="40">
+    <row r="41" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="C41" s="26" t="e" vm="41">
         <v>#VALUE!</v>
       </c>
       <c r="D41" s="27" t="s">
@@ -13479,9 +13660,13 @@
         <f t="array" aca="1" ref="K41" ca="1">_FV(C41,"Shares outstanding",TRUE)</f>
         <v>178718800</v>
       </c>
+      <c r="L41" t="str" cm="1">
+        <f t="array" aca="1" ref="L41" ca="1">_FV(C41,"Ticker symbol",TRUE)</f>
+        <v>LUNR</v>
+      </c>
     </row>
-    <row r="42" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C42" s="20" t="e" vm="41">
+    <row r="42" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="C42" s="20" t="e" vm="42">
         <v>#VALUE!</v>
       </c>
       <c r="D42" s="21" t="s">
@@ -13509,9 +13694,13 @@
         <f t="array" aca="1" ref="K42" ca="1">_FV(C42,"Shares outstanding",TRUE)</f>
         <v>345309400</v>
       </c>
+      <c r="L42" t="str" cm="1">
+        <f t="array" aca="1" ref="L42" ca="1">_FV(C42,"Ticker symbol",TRUE)</f>
+        <v>EVEX</v>
+      </c>
     </row>
-    <row r="43" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C43" s="26" t="e" vm="42">
+    <row r="43" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="C43" s="26" t="e" vm="43">
         <v>#VALUE!</v>
       </c>
       <c r="D43" s="27" t="s">
@@ -13539,9 +13728,13 @@
         <f t="array" aca="1" ref="K43" ca="1">_FV(C43,"Shares outstanding",TRUE)</f>
         <v>14923740</v>
       </c>
+      <c r="L43" t="str" cm="1">
+        <f t="array" aca="1" ref="L43" ca="1">_FV(C43,"Ticker symbol",TRUE)</f>
+        <v>DCO</v>
+      </c>
     </row>
-    <row r="44" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C44" s="20" t="e" vm="43">
+    <row r="44" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="C44" s="20" t="e" vm="44">
         <v>#VALUE!</v>
       </c>
       <c r="D44" s="21" t="s">
@@ -13569,9 +13762,13 @@
         <f t="array" aca="1" ref="K44" ca="1">_FV(C44,"Shares outstanding",TRUE)</f>
         <v>71984860</v>
       </c>
+      <c r="L44" t="str" cm="1">
+        <f t="array" aca="1" ref="L44" ca="1">_FV(C44,"Ticker symbol",TRUE)</f>
+        <v>EH</v>
+      </c>
     </row>
-    <row r="45" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C45" s="26" t="e" vm="44">
+    <row r="45" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="C45" s="26" t="e" vm="45">
         <v>#VALUE!</v>
       </c>
       <c r="D45" s="27" t="s">
@@ -13599,9 +13796,13 @@
         <f t="array" aca="1" ref="K45" ca="1">_FV(C45,"Shares outstanding",TRUE)</f>
         <v>144039900</v>
       </c>
+      <c r="L45" t="str" cm="1">
+        <f t="array" aca="1" ref="L45" ca="1">_FV(C45,"Ticker symbol",TRUE)</f>
+        <v>RDW</v>
+      </c>
     </row>
-    <row r="46" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C46" s="20" t="e" vm="45">
+    <row r="46" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="C46" s="20" t="e" vm="46">
         <v>#VALUE!</v>
       </c>
       <c r="D46" s="21" t="s">
@@ -13629,9 +13830,13 @@
         <f t="array" aca="1" ref="K46" ca="1">_FV(C46,"Shares outstanding",TRUE)</f>
         <v>35406240</v>
       </c>
+      <c r="L46" t="str" cm="1">
+        <f t="array" aca="1" ref="L46" ca="1">_FV(C46,"Ticker symbol",TRUE)</f>
+        <v>ATRO</v>
+      </c>
     </row>
-    <row r="47" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C47" s="26" t="e" vm="46">
+    <row r="47" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="C47" s="26" t="e" vm="47">
         <v>#VALUE!</v>
       </c>
       <c r="D47" s="27" t="s">
@@ -13659,9 +13864,13 @@
         <f t="array" aca="1" ref="K47" ca="1">_FV(C47,"Shares outstanding",TRUE)</f>
         <v>40663840</v>
       </c>
+      <c r="L47" t="str" cm="1">
+        <f t="array" aca="1" ref="L47" ca="1">_FV(C47,"Ticker symbol",TRUE)</f>
+        <v>CDRE</v>
+      </c>
     </row>
-    <row r="48" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C48" s="20" t="e" vm="47">
+    <row r="48" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="C48" s="20" t="e" vm="48">
         <v>#VALUE!</v>
       </c>
       <c r="D48" s="21" t="s">
@@ -13689,9 +13898,13 @@
         <f t="array" aca="1" ref="K48" ca="1">_FV(C48,"Shares outstanding",TRUE)</f>
         <v>99764260</v>
       </c>
+      <c r="L48" t="str" cm="1">
+        <f t="array" aca="1" ref="L48" ca="1">_FV(C48,"Ticker symbol",TRUE)</f>
+        <v>RCAT</v>
+      </c>
     </row>
-    <row r="49" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="C49" s="26" t="e" vm="48">
+    <row r="49" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="C49" s="26" t="e" vm="49">
         <v>#VALUE!</v>
       </c>
       <c r="D49" s="27" t="s">
@@ -13719,9 +13932,13 @@
         <f t="array" aca="1" ref="K49" ca="1">_FV(C49,"Shares outstanding",TRUE)</f>
         <v>7149530</v>
       </c>
+      <c r="L49" t="str" cm="1">
+        <f t="array" aca="1" ref="L49" ca="1">_FV(C49,"Ticker symbol",TRUE)</f>
+        <v>NPK</v>
+      </c>
     </row>
-    <row r="50" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="C50" s="20" t="e" vm="49">
+    <row r="50" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="C50" s="20" t="e" vm="50">
         <v>#VALUE!</v>
       </c>
       <c r="D50" s="21" t="s">
@@ -13749,9 +13966,13 @@
         <f t="array" aca="1" ref="K50" ca="1">_FV(C50,"Shares outstanding",TRUE)</f>
         <v>27421100</v>
       </c>
+      <c r="L50" t="str" cm="1">
+        <f t="array" aca="1" ref="L50" ca="1">_FV(C50,"Ticker symbol",TRUE)</f>
+        <v>AIRO</v>
+      </c>
     </row>
-    <row r="51" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="C51" s="26" t="e" vm="50">
+    <row r="51" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="C51" s="26" t="e" vm="51">
         <v>#VALUE!</v>
       </c>
       <c r="D51" s="27" t="s">
@@ -13779,9 +14000,13 @@
         <f t="array" aca="1" ref="K51" ca="1">_FV(C51,"Shares outstanding",TRUE)</f>
         <v>16162030</v>
       </c>
+      <c r="L51" t="str" cm="1">
+        <f t="array" aca="1" ref="L51" ca="1">_FV(C51,"Ticker symbol",TRUE)</f>
+        <v>RGR</v>
+      </c>
     </row>
-    <row r="52" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="C52" s="20" t="e" vm="51">
+    <row r="52" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="C52" s="20" t="e" vm="52">
         <v>#VALUE!</v>
       </c>
       <c r="D52" s="21" t="s">
@@ -13809,9 +14034,13 @@
         <f t="array" aca="1" ref="K52" ca="1">_FV(C52,"Shares outstanding",TRUE)</f>
         <v>98477720</v>
       </c>
+      <c r="L52" t="str" cm="1">
+        <f t="array" aca="1" ref="L52" ca="1">_FV(C52,"Ticker symbol",TRUE)</f>
+        <v>EVTL</v>
+      </c>
     </row>
-    <row r="53" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="C53" s="26" t="e" vm="52">
+    <row r="53" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="C53" s="26" t="e" vm="53">
         <v>#VALUE!</v>
       </c>
       <c r="D53" s="27" t="s">
@@ -13839,9 +14068,13 @@
         <f t="array" aca="1" ref="K53" ca="1">_FV(C53,"Shares outstanding",TRUE)</f>
         <v>12898580</v>
       </c>
+      <c r="L53" t="str" cm="1">
+        <f t="array" aca="1" ref="L53" ca="1">_FV(C53,"Ticker symbol",TRUE)</f>
+        <v>TATT</v>
+      </c>
     </row>
-    <row r="54" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="C54" s="20" t="e" vm="53">
+    <row r="54" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="C54" s="20" t="e" vm="54">
         <v>#VALUE!</v>
       </c>
       <c r="D54" s="21" t="s">
@@ -13869,9 +14102,13 @@
         <f t="array" aca="1" ref="K54" ca="1">_FV(C54,"Shares outstanding",TRUE)</f>
         <v>22703810</v>
       </c>
+      <c r="L54" t="str" cm="1">
+        <f t="array" aca="1" ref="L54" ca="1">_FV(C54,"Ticker symbol",TRUE)</f>
+        <v>BYRN</v>
+      </c>
     </row>
-    <row r="55" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="C55" s="26" t="e" vm="54">
+    <row r="55" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="C55" s="26" t="e" vm="55">
         <v>#VALUE!</v>
       </c>
       <c r="D55" s="27" t="s">
@@ -13899,9 +14136,13 @@
         <f t="array" aca="1" ref="K55" ca="1">_FV(C55,"Shares outstanding",TRUE)</f>
         <v>19855840</v>
       </c>
+      <c r="L55" t="str" cm="1">
+        <f t="array" aca="1" ref="L55" ca="1">_FV(C55,"Ticker symbol",TRUE)</f>
+        <v>PKE</v>
+      </c>
     </row>
-    <row r="56" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="C56" s="20" t="e" vm="55">
+    <row r="56" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="C56" s="20" t="e" vm="56">
         <v>#VALUE!</v>
       </c>
       <c r="D56" s="21" t="s">
@@ -13929,9 +14170,13 @@
         <f t="array" aca="1" ref="K56" ca="1">_FV(C56,"Shares outstanding",TRUE)</f>
         <v>105568300</v>
       </c>
+      <c r="L56" t="str" cm="1">
+        <f t="array" aca="1" ref="L56" ca="1">_FV(C56,"Ticker symbol",TRUE)</f>
+        <v>SATL</v>
+      </c>
     </row>
-    <row r="57" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="C57" s="26" t="e" vm="56">
+    <row r="57" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="C57" s="26" t="e" vm="57">
         <v>#VALUE!</v>
       </c>
       <c r="D57" s="27" t="s">
@@ -13959,9 +14204,13 @@
         <f t="array" aca="1" ref="K57" ca="1">_FV(C57,"Shares outstanding",TRUE)</f>
         <v>44310370</v>
       </c>
+      <c r="L57" t="str" cm="1">
+        <f t="array" aca="1" ref="L57" ca="1">_FV(C57,"Ticker symbol",TRUE)</f>
+        <v>SWBI</v>
+      </c>
     </row>
-    <row r="58" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="C58" s="20" t="e" vm="57">
+    <row r="58" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="C58" s="20" t="e" vm="58">
         <v>#VALUE!</v>
       </c>
       <c r="D58" s="21" t="s">
@@ -13989,9 +14238,13 @@
         <f t="array" aca="1" ref="K58" ca="1">_FV(C58,"Shares outstanding",TRUE)</f>
         <v>17628160</v>
       </c>
+      <c r="L58" t="str" cm="1">
+        <f t="array" aca="1" ref="L58" ca="1">_FV(C58,"Ticker symbol",TRUE)</f>
+        <v>ISSC</v>
+      </c>
     </row>
-    <row r="59" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="C59" s="26" t="e" vm="58">
+    <row r="59" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="C59" s="26" t="e" vm="59">
         <v>#VALUE!</v>
       </c>
       <c r="D59" s="27" t="s">
@@ -14019,8 +14272,12 @@
         <f t="array" aca="1" ref="K59" ca="1">_FV(C59,"Shares outstanding",TRUE)</f>
         <v>57590960</v>
       </c>
+      <c r="L59" t="str" cm="1">
+        <f t="array" aca="1" ref="L59" ca="1">_FV(C59,"Ticker symbol",TRUE)</f>
+        <v>SPCE</v>
+      </c>
     </row>
-    <row r="60" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:12" x14ac:dyDescent="0.3">
       <c r="C60" s="20" t="s">
         <v>116</v>
       </c>
@@ -14049,9 +14306,13 @@
         <f t="array" ref="K60">_FV(C60,"Shares outstanding",TRUE)</f>
         <v>#VALUE!</v>
       </c>
+      <c r="L60" t="e" cm="1" vm="40">
+        <f t="array" ref="L60">_FV(C60,"Ticker symbol",TRUE)</f>
+        <v>#VALUE!</v>
+      </c>
     </row>
-    <row r="61" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="C61" s="26" t="e" vm="59">
+    <row r="61" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="C61" s="26" t="e" vm="60">
         <v>#VALUE!</v>
       </c>
       <c r="D61" s="27" t="s">
@@ -14079,8 +14340,12 @@
         <f t="array" aca="1" ref="K61" ca="1">_FV(C61,"Shares outstanding",TRUE)</f>
         <v>117110800</v>
       </c>
+      <c r="L61" t="str" cm="1">
+        <f t="array" aca="1" ref="L61" ca="1">_FV(C61,"Ticker symbol",TRUE)</f>
+        <v>POWW</v>
+      </c>
     </row>
-    <row r="62" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B62" s="17"/>
       <c r="C62" s="20" t="s">
         <v>121</v>
@@ -14110,9 +14375,13 @@
         <f t="array" ref="K62">_FV(C62,"Shares outstanding",TRUE)</f>
         <v>#VALUE!</v>
       </c>
+      <c r="L62" t="e" cm="1" vm="40">
+        <f t="array" ref="L62">_FV(C62,"Ticker symbol",TRUE)</f>
+        <v>#VALUE!</v>
+      </c>
     </row>
-    <row r="63" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="C63" s="26" t="e" vm="60">
+    <row r="63" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="C63" s="26" t="e" vm="61">
         <v>#VALUE!</v>
       </c>
       <c r="D63" s="27" t="s">
@@ -14140,9 +14409,13 @@
         <f t="array" aca="1" ref="K63" ca="1">_FV(C63,"Shares outstanding",TRUE)</f>
         <v>16168350</v>
       </c>
+      <c r="L63" t="str" cm="1">
+        <f t="array" aca="1" ref="L63" ca="1">_FV(C63,"Ticker symbol",TRUE)</f>
+        <v>SPAI</v>
+      </c>
     </row>
-    <row r="64" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="C64" s="20" t="e" vm="61">
+    <row r="64" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="C64" s="20" t="e" vm="62">
         <v>#VALUE!</v>
       </c>
       <c r="D64" s="21" t="s">
@@ -14170,9 +14443,13 @@
         <f t="array" aca="1" ref="K64" ca="1">_FV(C64,"Shares outstanding",TRUE)</f>
         <v>18099350</v>
       </c>
+      <c r="L64" t="str" cm="1">
+        <f t="array" aca="1" ref="L64" ca="1">_FV(C64,"Ticker symbol",TRUE)</f>
+        <v>DPRO</v>
+      </c>
     </row>
-    <row r="65" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C65" s="26" t="e" vm="62">
+    <row r="65" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="C65" s="26" t="e" vm="63">
         <v>#VALUE!</v>
       </c>
       <c r="D65" s="27" t="s">
@@ -14200,9 +14477,13 @@
         <f t="array" aca="1" ref="K65" ca="1">_FV(C65,"Shares outstanding",TRUE)</f>
         <v>11248870</v>
       </c>
+      <c r="L65" t="str" cm="1">
+        <f t="array" aca="1" ref="L65" ca="1">_FV(C65,"Ticker symbol",TRUE)</f>
+        <v>CODA</v>
+      </c>
     </row>
-    <row r="66" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C66" s="20" t="e" vm="63">
+    <row r="66" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="C66" s="20" t="e" vm="64">
         <v>#VALUE!</v>
       </c>
       <c r="D66" s="21" t="s">
@@ -14230,9 +14511,13 @@
         <f t="array" aca="1" ref="K66" ca="1">_FV(C66,"Shares outstanding",TRUE)</f>
         <v>6913620</v>
       </c>
+      <c r="L66" t="str" cm="1">
+        <f t="array" aca="1" ref="L66" ca="1">_FV(C66,"Ticker symbol",TRUE)</f>
+        <v>OPXS</v>
+      </c>
     </row>
-    <row r="67" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C67" s="26" t="e" vm="64">
+    <row r="67" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="C67" s="26" t="e" vm="65">
         <v>#VALUE!</v>
       </c>
       <c r="D67" s="27" t="s">
@@ -14260,9 +14545,13 @@
         <f t="array" aca="1" ref="K67" ca="1">_FV(C67,"Shares outstanding",TRUE)</f>
         <v>31385150</v>
       </c>
+      <c r="L67" t="str" cm="1">
+        <f t="array" aca="1" ref="L67" ca="1">_FV(C67,"Ticker symbol",TRUE)</f>
+        <v>HOVR</v>
+      </c>
     </row>
-    <row r="68" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C68" s="20" t="e" vm="65">
+    <row r="68" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="C68" s="20" t="e" vm="66">
         <v>#VALUE!</v>
       </c>
       <c r="D68" s="21" t="s">
@@ -14290,9 +14579,13 @@
         <f t="array" aca="1" ref="K68" ca="1">_FV(C68,"Shares outstanding",TRUE)</f>
         <v>6180390</v>
       </c>
+      <c r="L68" t="str" cm="1">
+        <f t="array" aca="1" ref="L68" ca="1">_FV(C68,"Ticker symbol",TRUE)</f>
+        <v>SIF</v>
+      </c>
     </row>
-    <row r="69" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C69" s="26" t="e" vm="66">
+    <row r="69" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="C69" s="26" t="e" vm="67">
         <v>#VALUE!</v>
       </c>
       <c r="D69" s="27" t="s">
@@ -14320,9 +14613,13 @@
         <f t="array" aca="1" ref="K69" ca="1">_FV(C69,"Shares outstanding",TRUE)</f>
         <v>27260</v>
       </c>
+      <c r="L69" t="str" cm="1">
+        <f t="array" aca="1" ref="L69" ca="1">_FV(C69,"Ticker symbol",TRUE)</f>
+        <v>MOB</v>
+      </c>
     </row>
-    <row r="70" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C70" s="20" t="e" vm="67">
+    <row r="70" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="C70" s="20" t="e" vm="68">
         <v>#VALUE!</v>
       </c>
       <c r="D70" s="21" t="s">
@@ -14350,9 +14647,13 @@
         <f t="array" aca="1" ref="K70" ca="1">_FV(C70,"Shares outstanding",TRUE)</f>
         <v>20253320</v>
       </c>
+      <c r="L70" t="str" cm="1">
+        <f t="array" aca="1" ref="L70" ca="1">_FV(C70,"Ticker symbol",TRUE)</f>
+        <v>XTIA</v>
+      </c>
     </row>
-    <row r="71" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C71" s="26" t="e" vm="68">
+    <row r="71" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="C71" s="26" t="e" vm="69">
         <v>#VALUE!</v>
       </c>
       <c r="D71" s="27" t="s">
@@ -14380,9 +14681,13 @@
         <f t="array" aca="1" ref="K71" ca="1">_FV(C71,"Shares outstanding",TRUE)</f>
         <v>42267640</v>
       </c>
+      <c r="L71" t="str" cm="1">
+        <f t="array" aca="1" ref="L71" ca="1">_FV(C71,"Ticker symbol",TRUE)</f>
+        <v>KITT</v>
+      </c>
     </row>
-    <row r="72" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C72" s="20" t="e" vm="69">
+    <row r="72" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="C72" s="20" t="e" vm="70">
         <v>#VALUE!</v>
       </c>
       <c r="D72" s="21" t="s">
@@ -14410,9 +14715,13 @@
         <f t="array" aca="1" ref="K72" ca="1">_FV(C72,"Shares outstanding",TRUE)</f>
         <v>13030740</v>
       </c>
+      <c r="L72" t="str" cm="1">
+        <f t="array" aca="1" ref="L72" ca="1">_FV(C72,"Ticker symbol",TRUE)</f>
+        <v>CVU</v>
+      </c>
     </row>
-    <row r="73" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C73" s="26" t="e" vm="70">
+    <row r="73" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="C73" s="26" t="e" vm="71">
         <v>#VALUE!</v>
       </c>
       <c r="D73" s="27" t="s">
@@ -14440,9 +14749,13 @@
         <f t="array" aca="1" ref="K73" ca="1">_FV(C73,"Shares outstanding",TRUE)</f>
         <v>25447480</v>
       </c>
+      <c r="L73" t="str" cm="1">
+        <f t="array" aca="1" ref="L73" ca="1">_FV(C73,"Ticker symbol",TRUE)</f>
+        <v>SIDU</v>
+      </c>
     </row>
-    <row r="74" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C74" s="20" t="e" vm="71">
+    <row r="74" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="C74" s="20" t="e" vm="72">
         <v>#VALUE!</v>
       </c>
       <c r="D74" s="21" t="s">
@@ -14470,9 +14783,13 @@
         <f t="array" aca="1" ref="K74" ca="1">_FV(C74,"Shares outstanding",TRUE)</f>
         <v>18763630</v>
       </c>
+      <c r="L74" t="str" cm="1">
+        <f t="array" aca="1" ref="L74" ca="1">_FV(C74,"Ticker symbol",TRUE)</f>
+        <v>PRZO</v>
+      </c>
     </row>
-    <row r="75" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C75" s="26" t="e" vm="72">
+    <row r="75" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="C75" s="26" t="e" vm="73">
         <v>#VALUE!</v>
       </c>
       <c r="D75" s="27" t="s">
@@ -14500,9 +14817,13 @@
         <f t="array" aca="1" ref="K75" ca="1">_FV(C75,"Shares outstanding",TRUE)</f>
         <v>32144450</v>
       </c>
+      <c r="L75" t="str" cm="1">
+        <f t="array" aca="1" ref="L75" ca="1">_FV(C75,"Ticker symbol",TRUE)</f>
+        <v>GPUS</v>
+      </c>
     </row>
-    <row r="76" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C76" s="20" t="e" vm="73">
+    <row r="76" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="C76" s="20" t="e" vm="74">
         <v>#VALUE!</v>
       </c>
       <c r="D76" s="21" t="s">
@@ -14530,9 +14851,13 @@
         <f t="array" aca="1" ref="K76" ca="1">_FV(C76,"Shares outstanding",TRUE)</f>
         <v>11634370</v>
       </c>
+      <c r="L76" t="str" cm="1">
+        <f t="array" aca="1" ref="L76" ca="1">_FV(C76,"Ticker symbol",TRUE)</f>
+        <v>MNTS</v>
+      </c>
     </row>
-    <row r="77" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C77" s="26" t="e" vm="74">
+    <row r="77" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="C77" s="26" t="e" vm="75">
         <v>#VALUE!</v>
       </c>
       <c r="D77" s="27" t="s">
@@ -14559,6 +14884,10 @@
       <c r="K77" s="25" cm="1">
         <f t="array" aca="1" ref="K77" ca="1">_FV(C77,"Shares outstanding",TRUE)</f>
         <v>4771950</v>
+      </c>
+      <c r="L77" t="str" cm="1">
+        <f t="array" aca="1" ref="L77" ca="1">_FV(C77,"Ticker symbol",TRUE)</f>
+        <v>AIRI</v>
       </c>
     </row>
   </sheetData>
@@ -14690,7 +15019,7 @@
       </c>
     </row>
     <row r="2" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C2" s="3" t="e" vm="75">
+      <c r="C2" s="3" t="e" vm="76">
         <v>#VALUE!</v>
       </c>
       <c r="D2" s="4" t="s">
@@ -14720,7 +15049,7 @@
       </c>
     </row>
     <row r="3" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C3" s="8" t="e" vm="76">
+      <c r="C3" s="8" t="e" vm="77">
         <v>#VALUE!</v>
       </c>
       <c r="D3" s="9" t="s">
@@ -14750,7 +15079,7 @@
       </c>
     </row>
     <row r="4" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C4" s="3" t="e" vm="77">
+      <c r="C4" s="3" t="e" vm="78">
         <v>#VALUE!</v>
       </c>
       <c r="D4" s="4" t="s">
@@ -14780,7 +15109,7 @@
       </c>
     </row>
     <row r="5" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C5" s="8" t="e" vm="78">
+      <c r="C5" s="8" t="e" vm="79">
         <v>#VALUE!</v>
       </c>
       <c r="D5" s="9" t="s">
@@ -14810,7 +15139,7 @@
       </c>
     </row>
     <row r="6" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C6" s="3" t="e" vm="79">
+      <c r="C6" s="3" t="e" vm="80">
         <v>#VALUE!</v>
       </c>
       <c r="D6" s="4" t="s">
@@ -14840,7 +15169,7 @@
       </c>
     </row>
     <row r="7" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C7" s="8" t="e" vm="80">
+      <c r="C7" s="8" t="e" vm="81">
         <v>#VALUE!</v>
       </c>
       <c r="D7" s="9" t="s">
@@ -14870,7 +15199,7 @@
       </c>
     </row>
     <row r="8" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C8" s="3" t="e" vm="81">
+      <c r="C8" s="3" t="e" vm="82">
         <v>#VALUE!</v>
       </c>
       <c r="D8" s="4" t="s">
@@ -14900,7 +15229,7 @@
       </c>
     </row>
     <row r="9" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C9" s="8" t="e" vm="82">
+      <c r="C9" s="8" t="e" vm="83">
         <v>#VALUE!</v>
       </c>
       <c r="D9" s="9" t="s">
@@ -14930,7 +15259,7 @@
       </c>
     </row>
     <row r="10" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C10" s="3" t="e" vm="83">
+      <c r="C10" s="3" t="e" vm="84">
         <v>#VALUE!</v>
       </c>
       <c r="D10" s="4" t="s">
@@ -14960,7 +15289,7 @@
       </c>
     </row>
     <row r="11" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C11" s="8" t="e" vm="84">
+      <c r="C11" s="8" t="e" vm="85">
         <v>#VALUE!</v>
       </c>
       <c r="D11" s="9" t="s">
@@ -14990,7 +15319,7 @@
       </c>
     </row>
     <row r="12" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C12" s="3" t="e" vm="85">
+      <c r="C12" s="3" t="e" vm="86">
         <v>#VALUE!</v>
       </c>
       <c r="D12" s="4" t="s">
@@ -15020,7 +15349,7 @@
       </c>
     </row>
     <row r="13" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C13" s="8" t="e" vm="86">
+      <c r="C13" s="8" t="e" vm="87">
         <v>#VALUE!</v>
       </c>
       <c r="D13" s="9" t="s">
@@ -15050,7 +15379,7 @@
       </c>
     </row>
     <row r="14" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C14" s="3" t="e" vm="87">
+      <c r="C14" s="3" t="e" vm="88">
         <v>#VALUE!</v>
       </c>
       <c r="D14" s="4" t="s">
@@ -15080,7 +15409,7 @@
       </c>
     </row>
     <row r="15" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C15" s="8" t="e" vm="88">
+      <c r="C15" s="8" t="e" vm="89">
         <v>#VALUE!</v>
       </c>
       <c r="D15" s="9" t="s">
@@ -15110,7 +15439,7 @@
       </c>
     </row>
     <row r="16" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C16" s="3" t="e" vm="89">
+      <c r="C16" s="3" t="e" vm="90">
         <v>#VALUE!</v>
       </c>
       <c r="D16" s="4" t="s">
@@ -15140,7 +15469,7 @@
       </c>
     </row>
     <row r="17" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C17" s="8" t="e" vm="90">
+      <c r="C17" s="8" t="e" vm="91">
         <v>#VALUE!</v>
       </c>
       <c r="D17" s="9" t="s">
@@ -15170,7 +15499,7 @@
       </c>
     </row>
     <row r="18" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C18" s="3" t="e" vm="91">
+      <c r="C18" s="3" t="e" vm="92">
         <v>#VALUE!</v>
       </c>
       <c r="D18" s="4" t="s">
@@ -15200,7 +15529,7 @@
       </c>
     </row>
     <row r="19" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C19" s="8" t="e" vm="92">
+      <c r="C19" s="8" t="e" vm="93">
         <v>#VALUE!</v>
       </c>
       <c r="D19" s="9" t="s">
@@ -15230,7 +15559,7 @@
       </c>
     </row>
     <row r="20" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C20" s="3" t="e" vm="93">
+      <c r="C20" s="3" t="e" vm="94">
         <v>#VALUE!</v>
       </c>
       <c r="D20" s="4" t="s">
@@ -15260,7 +15589,7 @@
       </c>
     </row>
     <row r="21" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C21" s="8" t="e" vm="94">
+      <c r="C21" s="8" t="e" vm="95">
         <v>#VALUE!</v>
       </c>
       <c r="D21" s="9" t="s">
@@ -15290,7 +15619,7 @@
       </c>
     </row>
     <row r="22" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C22" s="3" t="e" vm="95">
+      <c r="C22" s="3" t="e" vm="96">
         <v>#VALUE!</v>
       </c>
       <c r="D22" s="4" t="s">
@@ -15320,7 +15649,7 @@
       </c>
     </row>
     <row r="23" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C23" s="8" t="e" vm="96">
+      <c r="C23" s="8" t="e" vm="97">
         <v>#VALUE!</v>
       </c>
       <c r="D23" s="9" t="s">
@@ -15350,7 +15679,7 @@
       </c>
     </row>
     <row r="24" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C24" s="3" t="e" vm="97">
+      <c r="C24" s="3" t="e" vm="98">
         <v>#VALUE!</v>
       </c>
       <c r="D24" s="4" t="s">
@@ -15380,7 +15709,7 @@
       </c>
     </row>
     <row r="25" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C25" s="8" t="e" vm="98">
+      <c r="C25" s="8" t="e" vm="99">
         <v>#VALUE!</v>
       </c>
       <c r="D25" s="9" t="s">
@@ -15410,7 +15739,7 @@
       </c>
     </row>
     <row r="26" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C26" s="3" t="e" vm="99">
+      <c r="C26" s="3" t="e" vm="100">
         <v>#VALUE!</v>
       </c>
       <c r="D26" s="4" t="s">
@@ -15440,7 +15769,7 @@
       </c>
     </row>
     <row r="27" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C27" s="8" t="e" vm="100">
+      <c r="C27" s="8" t="e" vm="101">
         <v>#VALUE!</v>
       </c>
       <c r="D27" s="9" t="s">
@@ -15470,7 +15799,7 @@
       </c>
     </row>
     <row r="28" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C28" s="3" t="e" vm="101">
+      <c r="C28" s="3" t="e" vm="102">
         <v>#VALUE!</v>
       </c>
       <c r="D28" s="4" t="s">
@@ -15500,7 +15829,7 @@
       </c>
     </row>
     <row r="29" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C29" s="8" t="e" vm="102">
+      <c r="C29" s="8" t="e" vm="103">
         <v>#VALUE!</v>
       </c>
       <c r="D29" s="9" t="s">
@@ -15530,7 +15859,7 @@
       </c>
     </row>
     <row r="30" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C30" s="3" t="e" vm="103">
+      <c r="C30" s="3" t="e" vm="104">
         <v>#VALUE!</v>
       </c>
       <c r="D30" s="4" t="s">
@@ -15560,7 +15889,7 @@
       </c>
     </row>
     <row r="31" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C31" s="8" t="e" vm="104">
+      <c r="C31" s="8" t="e" vm="105">
         <v>#VALUE!</v>
       </c>
       <c r="D31" s="9" t="s">
@@ -15590,7 +15919,7 @@
       </c>
     </row>
     <row r="32" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C32" s="3" t="e" vm="105">
+      <c r="C32" s="3" t="e" vm="106">
         <v>#VALUE!</v>
       </c>
       <c r="D32" s="4" t="s">
@@ -15620,7 +15949,7 @@
       </c>
     </row>
     <row r="33" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C33" s="8" t="e" vm="106">
+      <c r="C33" s="8" t="e" vm="107">
         <v>#VALUE!</v>
       </c>
       <c r="D33" s="9" t="s">
@@ -15650,7 +15979,7 @@
       </c>
     </row>
     <row r="34" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C34" s="3" t="e" vm="107">
+      <c r="C34" s="3" t="e" vm="108">
         <v>#VALUE!</v>
       </c>
       <c r="D34" s="4" t="s">
@@ -15680,7 +16009,7 @@
       </c>
     </row>
     <row r="35" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C35" s="8" t="e" vm="108">
+      <c r="C35" s="8" t="e" vm="109">
         <v>#VALUE!</v>
       </c>
       <c r="D35" s="9" t="s">
@@ -15710,7 +16039,7 @@
       </c>
     </row>
     <row r="36" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C36" s="3" t="e" vm="109">
+      <c r="C36" s="3" t="e" vm="110">
         <v>#VALUE!</v>
       </c>
       <c r="D36" s="4" t="s">
@@ -15740,7 +16069,7 @@
       </c>
     </row>
     <row r="37" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C37" s="8" t="e" vm="110">
+      <c r="C37" s="8" t="e" vm="111">
         <v>#VALUE!</v>
       </c>
       <c r="D37" s="9" t="s">
@@ -15770,7 +16099,7 @@
       </c>
     </row>
     <row r="38" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C38" s="3" t="e" vm="111">
+      <c r="C38" s="3" t="e" vm="112">
         <v>#VALUE!</v>
       </c>
       <c r="D38" s="4" t="s">
@@ -15800,7 +16129,7 @@
       </c>
     </row>
     <row r="39" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C39" s="8" t="e" vm="112">
+      <c r="C39" s="8" t="e" vm="113">
         <v>#VALUE!</v>
       </c>
       <c r="D39" s="9" t="s">
@@ -15830,7 +16159,7 @@
       </c>
     </row>
     <row r="40" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C40" s="3" t="e" vm="113">
+      <c r="C40" s="3" t="e" vm="114">
         <v>#VALUE!</v>
       </c>
       <c r="D40" s="4" t="s">
@@ -15860,7 +16189,7 @@
       </c>
     </row>
     <row r="41" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C41" s="8" t="e" vm="114">
+      <c r="C41" s="8" t="e" vm="115">
         <v>#VALUE!</v>
       </c>
       <c r="D41" s="9" t="s">
@@ -15890,7 +16219,7 @@
       </c>
     </row>
     <row r="42" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C42" s="3" t="e" vm="115">
+      <c r="C42" s="3" t="e" vm="116">
         <v>#VALUE!</v>
       </c>
       <c r="D42" s="4" t="s">
@@ -15920,7 +16249,7 @@
       </c>
     </row>
     <row r="43" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C43" s="8" t="e" vm="116">
+      <c r="C43" s="8" t="e" vm="117">
         <v>#VALUE!</v>
       </c>
       <c r="D43" s="9" t="s">
@@ -15950,7 +16279,7 @@
       </c>
     </row>
     <row r="44" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C44" s="3" t="e" vm="117">
+      <c r="C44" s="3" t="e" vm="118">
         <v>#VALUE!</v>
       </c>
       <c r="D44" s="4" t="s">
@@ -15980,7 +16309,7 @@
       </c>
     </row>
     <row r="45" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C45" s="8" t="e" vm="118">
+      <c r="C45" s="8" t="e" vm="119">
         <v>#VALUE!</v>
       </c>
       <c r="D45" s="9" t="s">
@@ -16010,7 +16339,7 @@
       </c>
     </row>
     <row r="46" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C46" s="3" t="e" vm="119">
+      <c r="C46" s="3" t="e" vm="120">
         <v>#VALUE!</v>
       </c>
       <c r="D46" s="4" t="s">
@@ -16040,7 +16369,7 @@
       </c>
     </row>
     <row r="47" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C47" s="8" t="e" vm="120">
+      <c r="C47" s="8" t="e" vm="121">
         <v>#VALUE!</v>
       </c>
       <c r="D47" s="9" t="s">
@@ -16070,7 +16399,7 @@
       </c>
     </row>
     <row r="48" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C48" s="3" t="e" vm="121">
+      <c r="C48" s="3" t="e" vm="122">
         <v>#VALUE!</v>
       </c>
       <c r="D48" s="4" t="s">
@@ -16100,7 +16429,7 @@
       </c>
     </row>
     <row r="49" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C49" s="8" t="e" vm="122">
+      <c r="C49" s="8" t="e" vm="123">
         <v>#VALUE!</v>
       </c>
       <c r="D49" s="9" t="s">
@@ -16130,7 +16459,7 @@
       </c>
     </row>
     <row r="50" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C50" s="3" t="e" vm="123">
+      <c r="C50" s="3" t="e" vm="124">
         <v>#VALUE!</v>
       </c>
       <c r="D50" s="4" t="s">
@@ -16160,7 +16489,7 @@
       </c>
     </row>
     <row r="51" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C51" s="8" t="e" vm="124">
+      <c r="C51" s="8" t="e" vm="125">
         <v>#VALUE!</v>
       </c>
       <c r="D51" s="9" t="s">
@@ -16190,7 +16519,7 @@
       </c>
     </row>
     <row r="52" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C52" s="3" t="e" vm="125">
+      <c r="C52" s="3" t="e" vm="126">
         <v>#VALUE!</v>
       </c>
       <c r="D52" s="4" t="s">
@@ -16220,7 +16549,7 @@
       </c>
     </row>
     <row r="53" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C53" s="8" t="e" vm="126">
+      <c r="C53" s="8" t="e" vm="127">
         <v>#VALUE!</v>
       </c>
       <c r="D53" s="9" t="s">
@@ -16250,7 +16579,7 @@
       </c>
     </row>
     <row r="54" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C54" s="3" t="e" vm="127">
+      <c r="C54" s="3" t="e" vm="128">
         <v>#VALUE!</v>
       </c>
       <c r="D54" s="4" t="s">
@@ -16280,7 +16609,7 @@
       </c>
     </row>
     <row r="55" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C55" s="8" t="e" vm="128">
+      <c r="C55" s="8" t="e" vm="129">
         <v>#VALUE!</v>
       </c>
       <c r="D55" s="9" t="s">
@@ -16340,7 +16669,7 @@
       </c>
     </row>
     <row r="57" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C57" s="8" t="e" vm="129">
+      <c r="C57" s="8" t="e" vm="130">
         <v>#VALUE!</v>
       </c>
       <c r="D57" s="9" t="s">
@@ -16370,7 +16699,7 @@
       </c>
     </row>
     <row r="58" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C58" s="3" t="e" vm="130">
+      <c r="C58" s="3" t="e" vm="131">
         <v>#VALUE!</v>
       </c>
       <c r="D58" s="4" t="s">
@@ -16400,7 +16729,7 @@
       </c>
     </row>
     <row r="59" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C59" s="8" t="e" vm="131">
+      <c r="C59" s="8" t="e" vm="132">
         <v>#VALUE!</v>
       </c>
       <c r="D59" s="9" t="s">
@@ -16430,7 +16759,7 @@
       </c>
     </row>
     <row r="60" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C60" s="3" t="e" vm="132">
+      <c r="C60" s="3" t="e" vm="133">
         <v>#VALUE!</v>
       </c>
       <c r="D60" s="4" t="s">
@@ -16460,7 +16789,7 @@
       </c>
     </row>
     <row r="61" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C61" s="8" t="e" vm="133">
+      <c r="C61" s="8" t="e" vm="134">
         <v>#VALUE!</v>
       </c>
       <c r="D61" s="9" t="s">
@@ -16490,7 +16819,7 @@
       </c>
     </row>
     <row r="62" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C62" s="3" t="e" vm="134">
+      <c r="C62" s="3" t="e" vm="135">
         <v>#VALUE!</v>
       </c>
       <c r="D62" s="4" t="s">
@@ -16520,7 +16849,7 @@
       </c>
     </row>
     <row r="63" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C63" s="8" t="e" vm="135">
+      <c r="C63" s="8" t="e" vm="136">
         <v>#VALUE!</v>
       </c>
       <c r="D63" s="9" t="s">
@@ -16550,7 +16879,7 @@
       </c>
     </row>
     <row r="64" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C64" s="3" t="e" vm="136">
+      <c r="C64" s="3" t="e" vm="137">
         <v>#VALUE!</v>
       </c>
       <c r="D64" s="4" t="s">
@@ -16580,7 +16909,7 @@
       </c>
     </row>
     <row r="65" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C65" s="8" t="e" vm="137">
+      <c r="C65" s="8" t="e" vm="138">
         <v>#VALUE!</v>
       </c>
       <c r="D65" s="9" t="s">
@@ -16610,7 +16939,7 @@
       </c>
     </row>
     <row r="66" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C66" s="3" t="e" vm="138">
+      <c r="C66" s="3" t="e" vm="139">
         <v>#VALUE!</v>
       </c>
       <c r="D66" s="4" t="s">
@@ -16640,7 +16969,7 @@
       </c>
     </row>
     <row r="67" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C67" s="8" t="e" vm="139">
+      <c r="C67" s="8" t="e" vm="140">
         <v>#VALUE!</v>
       </c>
       <c r="D67" s="9" t="s">
@@ -16670,7 +16999,7 @@
       </c>
     </row>
     <row r="68" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C68" s="3" t="e" vm="140">
+      <c r="C68" s="3" t="e" vm="141">
         <v>#VALUE!</v>
       </c>
       <c r="D68" s="4" t="s">
@@ -16700,7 +17029,7 @@
       </c>
     </row>
     <row r="69" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C69" s="8" t="e" vm="141">
+      <c r="C69" s="8" t="e" vm="142">
         <v>#VALUE!</v>
       </c>
       <c r="D69" s="9" t="s">
@@ -16730,7 +17059,7 @@
       </c>
     </row>
     <row r="70" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C70" s="3" t="e" vm="142">
+      <c r="C70" s="3" t="e" vm="143">
         <v>#VALUE!</v>
       </c>
       <c r="D70" s="4" t="s">
@@ -16760,7 +17089,7 @@
       </c>
     </row>
     <row r="71" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C71" s="8" t="e" vm="143">
+      <c r="C71" s="8" t="e" vm="144">
         <v>#VALUE!</v>
       </c>
       <c r="D71" s="9" t="s">
@@ -16790,7 +17119,7 @@
       </c>
     </row>
     <row r="72" spans="3:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C72" s="3" t="e" vm="144">
+      <c r="C72" s="3" t="e" vm="145">
         <v>#VALUE!</v>
       </c>
       <c r="D72" s="4" t="s">

</xml_diff>